<commit_message>
Add manual Out/New Count checkbox columns to Count Sheet
Richard requested two plain manual-tick columns on the Count Sheet tab:
"Out" (red) and "New Count" (green), with no automated logic behind
them. Inserted as columns I/J, shifting Counted kg/pcs, Var kg/pcs,
Reason and Notes from I-N to K-P. Reconciliation's Counted kg/pcs SUMIF
ranges (F/G, rows 5-18) are repointed at the new K/L columns to match.

Verified end-to-end with synthetic items via buildInventoryCountWorkbook
and a LibreOffice recalc (1087 formulas, 0 errors).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017SywvQLutU4oCcdV3fA2oE
</commit_message>
<xml_diff>
--- a/public/templates/inventory-count-template.xlsx
+++ b/public/templates/inventory-count-template.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -171,8 +171,14 @@
       <color rgb="FF595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1F3B2C"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -209,8 +215,18 @@
         <bgColor rgb="FFEDE7DC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -248,6 +264,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -259,7 +289,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -533,6 +563,12 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1293,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N161"/>
+  <dimension ref="A1:P161"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="46" min="1" max="1"/>
@@ -1304,7 +1340,8 @@
     <col width="10" customWidth="1" style="46" min="6" max="6"/>
     <col width="15" customWidth="1" style="46" min="7" max="7"/>
     <col width="10" customWidth="1" style="46" min="8" max="8"/>
-    <col width="11" customWidth="1" style="46" min="9" max="10"/>
+    <col width="9" customWidth="1" style="46" min="9" max="10"/>
+    <col width="11" customWidth="1" style="47" min="10" max="10"/>
     <col width="10" customWidth="1" style="46" min="11" max="11"/>
     <col width="9" customWidth="1" style="46" min="12" max="12"/>
     <col width="18" customWidth="1" style="46" min="13" max="13"/>
@@ -1368,30 +1405,40 @@
       </c>
       <c r="I4" s="58" t="inlineStr">
         <is>
+          <t>Out</t>
+        </is>
+      </c>
+      <c r="J4" s="58" t="inlineStr">
+        <is>
+          <t>New Count</t>
+        </is>
+      </c>
+      <c r="K4" s="58" t="inlineStr">
+        <is>
           <t>Counted kg</t>
         </is>
       </c>
-      <c r="J4" s="58" t="inlineStr">
+      <c r="L4" s="58" t="inlineStr">
         <is>
           <t>Counted pcs</t>
         </is>
       </c>
-      <c r="K4" s="58" t="inlineStr">
+      <c r="M4" s="58" t="inlineStr">
         <is>
           <t>Var kg</t>
         </is>
       </c>
-      <c r="L4" s="58" t="inlineStr">
+      <c r="N4" s="58" t="inlineStr">
         <is>
           <t>Var pcs</t>
         </is>
       </c>
-      <c r="M4" s="58" t="inlineStr">
+      <c r="O4" s="58" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="N4" s="58" t="inlineStr">
+      <c r="P4" s="58" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1405,18 +1452,20 @@
       <c r="E5" s="59" t="n"/>
       <c r="F5" s="60" t="n"/>
       <c r="G5" s="54" t="n"/>
-      <c r="I5" s="61" t="n"/>
-      <c r="J5" s="62" t="n"/>
-      <c r="K5" s="59">
-        <f>IF(I5="","",ROUND(I5-E5,2))</f>
-        <v/>
-      </c>
-      <c r="L5" s="60">
-        <f>IF(J5="","",J5-F5)</f>
-        <v/>
-      </c>
-      <c r="M5" s="56" t="n"/>
-      <c r="N5" s="56" t="n"/>
+      <c r="I5" s="92" t="n"/>
+      <c r="J5" s="93" t="n"/>
+      <c r="K5" s="61" t="n"/>
+      <c r="L5" s="62" t="n"/>
+      <c r="M5" s="59">
+        <f>IF(K5="","",ROUND(K5-E5,2))</f>
+        <v/>
+      </c>
+      <c r="N5" s="60">
+        <f>IF(L5="","",L5-F5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="56" t="n"/>
+      <c r="P5" s="56" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="47">
       <c r="A6" s="54" t="n"/>
@@ -1426,18 +1475,20 @@
       <c r="E6" s="59" t="n"/>
       <c r="F6" s="60" t="n"/>
       <c r="G6" s="54" t="n"/>
-      <c r="I6" s="61" t="n"/>
-      <c r="J6" s="62" t="n"/>
-      <c r="K6" s="59">
+      <c r="I6" s="92" t="n"/>
+      <c r="J6" s="93" t="n"/>
+      <c r="K6" s="61" t="n"/>
+      <c r="L6" s="62" t="n"/>
+      <c r="M6" s="59">
         <f>IF(I6="","",ROUND(I6-E6,2))</f>
         <v/>
       </c>
-      <c r="L6" s="60">
+      <c r="N6" s="60">
         <f>IF(J6="","",J6-F6)</f>
         <v/>
       </c>
-      <c r="M6" s="56" t="n"/>
-      <c r="N6" s="56" t="n"/>
+      <c r="O6" s="56" t="n"/>
+      <c r="P6" s="56" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="47">
       <c r="A7" s="54" t="n"/>
@@ -1447,18 +1498,20 @@
       <c r="E7" s="59" t="n"/>
       <c r="F7" s="60" t="n"/>
       <c r="G7" s="54" t="n"/>
-      <c r="I7" s="61" t="n"/>
-      <c r="J7" s="62" t="n"/>
-      <c r="K7" s="59">
+      <c r="I7" s="92" t="n"/>
+      <c r="J7" s="93" t="n"/>
+      <c r="K7" s="61" t="n"/>
+      <c r="L7" s="62" t="n"/>
+      <c r="M7" s="59">
         <f>IF(I7="","",ROUND(I7-E7,2))</f>
         <v/>
       </c>
-      <c r="L7" s="60">
+      <c r="N7" s="60">
         <f>IF(J7="","",J7-F7)</f>
         <v/>
       </c>
-      <c r="M7" s="56" t="n"/>
-      <c r="N7" s="56" t="n"/>
+      <c r="O7" s="56" t="n"/>
+      <c r="P7" s="56" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="47">
       <c r="A8" s="54" t="n"/>
@@ -1468,18 +1521,20 @@
       <c r="E8" s="59" t="n"/>
       <c r="F8" s="60" t="n"/>
       <c r="G8" s="54" t="n"/>
-      <c r="I8" s="61" t="n"/>
-      <c r="J8" s="62" t="n"/>
-      <c r="K8" s="59">
+      <c r="I8" s="92" t="n"/>
+      <c r="J8" s="93" t="n"/>
+      <c r="K8" s="61" t="n"/>
+      <c r="L8" s="62" t="n"/>
+      <c r="M8" s="59">
         <f>IF(I8="","",ROUND(I8-E8,2))</f>
         <v/>
       </c>
-      <c r="L8" s="60">
+      <c r="N8" s="60">
         <f>IF(J8="","",J8-F8)</f>
         <v/>
       </c>
-      <c r="M8" s="56" t="n"/>
-      <c r="N8" s="56" t="n"/>
+      <c r="O8" s="56" t="n"/>
+      <c r="P8" s="56" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="47">
       <c r="A9" s="54" t="n"/>
@@ -1489,18 +1544,20 @@
       <c r="E9" s="59" t="n"/>
       <c r="F9" s="60" t="n"/>
       <c r="G9" s="54" t="n"/>
-      <c r="I9" s="61" t="n"/>
-      <c r="J9" s="62" t="n"/>
-      <c r="K9" s="59">
+      <c r="I9" s="92" t="n"/>
+      <c r="J9" s="93" t="n"/>
+      <c r="K9" s="61" t="n"/>
+      <c r="L9" s="62" t="n"/>
+      <c r="M9" s="59">
         <f>IF(I9="","",ROUND(I9-E9,2))</f>
         <v/>
       </c>
-      <c r="L9" s="60">
+      <c r="N9" s="60">
         <f>IF(J9="","",J9-F9)</f>
         <v/>
       </c>
-      <c r="M9" s="56" t="n"/>
-      <c r="N9" s="56" t="n"/>
+      <c r="O9" s="56" t="n"/>
+      <c r="P9" s="56" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="47">
       <c r="A10" s="54" t="n"/>
@@ -1510,18 +1567,20 @@
       <c r="E10" s="59" t="n"/>
       <c r="F10" s="60" t="n"/>
       <c r="G10" s="54" t="n"/>
-      <c r="I10" s="61" t="n"/>
-      <c r="J10" s="62" t="n"/>
-      <c r="K10" s="59">
+      <c r="I10" s="92" t="n"/>
+      <c r="J10" s="93" t="n"/>
+      <c r="K10" s="61" t="n"/>
+      <c r="L10" s="62" t="n"/>
+      <c r="M10" s="59">
         <f>IF(I10="","",ROUND(I10-E10,2))</f>
         <v/>
       </c>
-      <c r="L10" s="60">
+      <c r="N10" s="60">
         <f>IF(J10="","",J10-F10)</f>
         <v/>
       </c>
-      <c r="M10" s="56" t="n"/>
-      <c r="N10" s="56" t="n"/>
+      <c r="O10" s="56" t="n"/>
+      <c r="P10" s="56" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="47">
       <c r="A11" s="54" t="n"/>
@@ -1531,18 +1590,20 @@
       <c r="E11" s="59" t="n"/>
       <c r="F11" s="60" t="n"/>
       <c r="G11" s="54" t="n"/>
-      <c r="I11" s="61" t="n"/>
-      <c r="J11" s="62" t="n"/>
-      <c r="K11" s="59">
+      <c r="I11" s="92" t="n"/>
+      <c r="J11" s="93" t="n"/>
+      <c r="K11" s="61" t="n"/>
+      <c r="L11" s="62" t="n"/>
+      <c r="M11" s="59">
         <f>IF(I11="","",ROUND(I11-E11,2))</f>
         <v/>
       </c>
-      <c r="L11" s="60">
+      <c r="N11" s="60">
         <f>IF(J11="","",J11-F11)</f>
         <v/>
       </c>
-      <c r="M11" s="56" t="n"/>
-      <c r="N11" s="56" t="n"/>
+      <c r="O11" s="56" t="n"/>
+      <c r="P11" s="56" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="47">
       <c r="A12" s="54" t="n"/>
@@ -1552,18 +1613,20 @@
       <c r="E12" s="59" t="n"/>
       <c r="F12" s="60" t="n"/>
       <c r="G12" s="54" t="n"/>
-      <c r="I12" s="61" t="n"/>
-      <c r="J12" s="62" t="n"/>
-      <c r="K12" s="59">
+      <c r="I12" s="92" t="n"/>
+      <c r="J12" s="93" t="n"/>
+      <c r="K12" s="61" t="n"/>
+      <c r="L12" s="62" t="n"/>
+      <c r="M12" s="59">
         <f>IF(I12="","",ROUND(I12-E12,2))</f>
         <v/>
       </c>
-      <c r="L12" s="60">
+      <c r="N12" s="60">
         <f>IF(J12="","",J12-F12)</f>
         <v/>
       </c>
-      <c r="M12" s="56" t="n"/>
-      <c r="N12" s="56" t="n"/>
+      <c r="O12" s="56" t="n"/>
+      <c r="P12" s="56" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="47">
       <c r="A13" s="54" t="n"/>
@@ -1573,18 +1636,20 @@
       <c r="E13" s="59" t="n"/>
       <c r="F13" s="60" t="n"/>
       <c r="G13" s="54" t="n"/>
-      <c r="I13" s="61" t="n"/>
-      <c r="J13" s="62" t="n"/>
-      <c r="K13" s="59">
+      <c r="I13" s="92" t="n"/>
+      <c r="J13" s="93" t="n"/>
+      <c r="K13" s="61" t="n"/>
+      <c r="L13" s="62" t="n"/>
+      <c r="M13" s="59">
         <f>IF(I13="","",ROUND(I13-E13,2))</f>
         <v/>
       </c>
-      <c r="L13" s="60">
+      <c r="N13" s="60">
         <f>IF(J13="","",J13-F13)</f>
         <v/>
       </c>
-      <c r="M13" s="56" t="n"/>
-      <c r="N13" s="56" t="n"/>
+      <c r="O13" s="56" t="n"/>
+      <c r="P13" s="56" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="47">
       <c r="A14" s="54" t="n"/>
@@ -1594,18 +1659,20 @@
       <c r="E14" s="59" t="n"/>
       <c r="F14" s="60" t="n"/>
       <c r="G14" s="54" t="n"/>
-      <c r="I14" s="61" t="n"/>
-      <c r="J14" s="62" t="n"/>
-      <c r="K14" s="59">
+      <c r="I14" s="92" t="n"/>
+      <c r="J14" s="93" t="n"/>
+      <c r="K14" s="61" t="n"/>
+      <c r="L14" s="62" t="n"/>
+      <c r="M14" s="59">
         <f>IF(I14="","",ROUND(I14-E14,2))</f>
         <v/>
       </c>
-      <c r="L14" s="60">
+      <c r="N14" s="60">
         <f>IF(J14="","",J14-F14)</f>
         <v/>
       </c>
-      <c r="M14" s="56" t="n"/>
-      <c r="N14" s="56" t="n"/>
+      <c r="O14" s="56" t="n"/>
+      <c r="P14" s="56" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="47">
       <c r="A15" s="54" t="n"/>
@@ -1615,18 +1682,20 @@
       <c r="E15" s="59" t="n"/>
       <c r="F15" s="60" t="n"/>
       <c r="G15" s="54" t="n"/>
-      <c r="I15" s="61" t="n"/>
-      <c r="J15" s="62" t="n"/>
-      <c r="K15" s="59">
+      <c r="I15" s="92" t="n"/>
+      <c r="J15" s="93" t="n"/>
+      <c r="K15" s="61" t="n"/>
+      <c r="L15" s="62" t="n"/>
+      <c r="M15" s="59">
         <f>IF(I15="","",ROUND(I15-E15,2))</f>
         <v/>
       </c>
-      <c r="L15" s="60">
+      <c r="N15" s="60">
         <f>IF(J15="","",J15-F15)</f>
         <v/>
       </c>
-      <c r="M15" s="56" t="n"/>
-      <c r="N15" s="56" t="n"/>
+      <c r="O15" s="56" t="n"/>
+      <c r="P15" s="56" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="47">
       <c r="A16" s="54" t="n"/>
@@ -1636,18 +1705,20 @@
       <c r="E16" s="59" t="n"/>
       <c r="F16" s="60" t="n"/>
       <c r="G16" s="54" t="n"/>
-      <c r="I16" s="61" t="n"/>
-      <c r="J16" s="62" t="n"/>
-      <c r="K16" s="59">
+      <c r="I16" s="92" t="n"/>
+      <c r="J16" s="93" t="n"/>
+      <c r="K16" s="61" t="n"/>
+      <c r="L16" s="62" t="n"/>
+      <c r="M16" s="59">
         <f>IF(I16="","",ROUND(I16-E16,2))</f>
         <v/>
       </c>
-      <c r="L16" s="60">
+      <c r="N16" s="60">
         <f>IF(J16="","",J16-F16)</f>
         <v/>
       </c>
-      <c r="M16" s="56" t="n"/>
-      <c r="N16" s="56" t="n"/>
+      <c r="O16" s="56" t="n"/>
+      <c r="P16" s="56" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="47">
       <c r="A17" s="54" t="n"/>
@@ -1657,18 +1728,20 @@
       <c r="E17" s="59" t="n"/>
       <c r="F17" s="60" t="n"/>
       <c r="G17" s="54" t="n"/>
-      <c r="I17" s="61" t="n"/>
-      <c r="J17" s="62" t="n"/>
-      <c r="K17" s="59">
+      <c r="I17" s="92" t="n"/>
+      <c r="J17" s="93" t="n"/>
+      <c r="K17" s="61" t="n"/>
+      <c r="L17" s="62" t="n"/>
+      <c r="M17" s="59">
         <f>IF(I17="","",ROUND(I17-E17,2))</f>
         <v/>
       </c>
-      <c r="L17" s="60">
+      <c r="N17" s="60">
         <f>IF(J17="","",J17-F17)</f>
         <v/>
       </c>
-      <c r="M17" s="56" t="n"/>
-      <c r="N17" s="56" t="n"/>
+      <c r="O17" s="56" t="n"/>
+      <c r="P17" s="56" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="47">
       <c r="A18" s="54" t="n"/>
@@ -1678,18 +1751,20 @@
       <c r="E18" s="59" t="n"/>
       <c r="F18" s="60" t="n"/>
       <c r="G18" s="54" t="n"/>
-      <c r="I18" s="61" t="n"/>
-      <c r="J18" s="62" t="n"/>
-      <c r="K18" s="59">
+      <c r="I18" s="92" t="n"/>
+      <c r="J18" s="93" t="n"/>
+      <c r="K18" s="61" t="n"/>
+      <c r="L18" s="62" t="n"/>
+      <c r="M18" s="59">
         <f>IF(I18="","",ROUND(I18-E18,2))</f>
         <v/>
       </c>
-      <c r="L18" s="60">
+      <c r="N18" s="60">
         <f>IF(J18="","",J18-F18)</f>
         <v/>
       </c>
-      <c r="M18" s="56" t="n"/>
-      <c r="N18" s="56" t="n"/>
+      <c r="O18" s="56" t="n"/>
+      <c r="P18" s="56" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="47">
       <c r="A19" s="54" t="n"/>
@@ -1699,18 +1774,20 @@
       <c r="E19" s="59" t="n"/>
       <c r="F19" s="60" t="n"/>
       <c r="G19" s="54" t="n"/>
-      <c r="I19" s="61" t="n"/>
-      <c r="J19" s="62" t="n"/>
-      <c r="K19" s="59">
+      <c r="I19" s="92" t="n"/>
+      <c r="J19" s="93" t="n"/>
+      <c r="K19" s="61" t="n"/>
+      <c r="L19" s="62" t="n"/>
+      <c r="M19" s="59">
         <f>IF(I19="","",ROUND(I19-E19,2))</f>
         <v/>
       </c>
-      <c r="L19" s="60">
+      <c r="N19" s="60">
         <f>IF(J19="","",J19-F19)</f>
         <v/>
       </c>
-      <c r="M19" s="56" t="n"/>
-      <c r="N19" s="56" t="n"/>
+      <c r="O19" s="56" t="n"/>
+      <c r="P19" s="56" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="47">
       <c r="A20" s="54" t="n"/>
@@ -1720,18 +1797,20 @@
       <c r="E20" s="59" t="n"/>
       <c r="F20" s="60" t="n"/>
       <c r="G20" s="54" t="n"/>
-      <c r="I20" s="61" t="n"/>
-      <c r="J20" s="62" t="n"/>
-      <c r="K20" s="59">
+      <c r="I20" s="92" t="n"/>
+      <c r="J20" s="93" t="n"/>
+      <c r="K20" s="61" t="n"/>
+      <c r="L20" s="62" t="n"/>
+      <c r="M20" s="59">
         <f>IF(I20="","",ROUND(I20-E20,2))</f>
         <v/>
       </c>
-      <c r="L20" s="60">
+      <c r="N20" s="60">
         <f>IF(J20="","",J20-F20)</f>
         <v/>
       </c>
-      <c r="M20" s="56" t="n"/>
-      <c r="N20" s="56" t="n"/>
+      <c r="O20" s="56" t="n"/>
+      <c r="P20" s="56" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="47">
       <c r="A21" s="54" t="n"/>
@@ -1741,18 +1820,20 @@
       <c r="E21" s="59" t="n"/>
       <c r="F21" s="60" t="n"/>
       <c r="G21" s="54" t="n"/>
-      <c r="I21" s="61" t="n"/>
-      <c r="J21" s="62" t="n"/>
-      <c r="K21" s="59">
+      <c r="I21" s="92" t="n"/>
+      <c r="J21" s="93" t="n"/>
+      <c r="K21" s="61" t="n"/>
+      <c r="L21" s="62" t="n"/>
+      <c r="M21" s="59">
         <f>IF(I21="","",ROUND(I21-E21,2))</f>
         <v/>
       </c>
-      <c r="L21" s="60">
+      <c r="N21" s="60">
         <f>IF(J21="","",J21-F21)</f>
         <v/>
       </c>
-      <c r="M21" s="56" t="n"/>
-      <c r="N21" s="56" t="n"/>
+      <c r="O21" s="56" t="n"/>
+      <c r="P21" s="56" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="47">
       <c r="A22" s="54" t="n"/>
@@ -1762,18 +1843,20 @@
       <c r="E22" s="59" t="n"/>
       <c r="F22" s="60" t="n"/>
       <c r="G22" s="54" t="n"/>
-      <c r="I22" s="61" t="n"/>
-      <c r="J22" s="62" t="n"/>
-      <c r="K22" s="59">
+      <c r="I22" s="92" t="n"/>
+      <c r="J22" s="93" t="n"/>
+      <c r="K22" s="61" t="n"/>
+      <c r="L22" s="62" t="n"/>
+      <c r="M22" s="59">
         <f>IF(I22="","",ROUND(I22-E22,2))</f>
         <v/>
       </c>
-      <c r="L22" s="60">
+      <c r="N22" s="60">
         <f>IF(J22="","",J22-F22)</f>
         <v/>
       </c>
-      <c r="M22" s="56" t="n"/>
-      <c r="N22" s="56" t="n"/>
+      <c r="O22" s="56" t="n"/>
+      <c r="P22" s="56" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="47">
       <c r="A23" s="54" t="n"/>
@@ -1783,18 +1866,20 @@
       <c r="E23" s="59" t="n"/>
       <c r="F23" s="60" t="n"/>
       <c r="G23" s="54" t="n"/>
-      <c r="I23" s="61" t="n"/>
-      <c r="J23" s="62" t="n"/>
-      <c r="K23" s="59">
+      <c r="I23" s="92" t="n"/>
+      <c r="J23" s="93" t="n"/>
+      <c r="K23" s="61" t="n"/>
+      <c r="L23" s="62" t="n"/>
+      <c r="M23" s="59">
         <f>IF(I23="","",ROUND(I23-E23,2))</f>
         <v/>
       </c>
-      <c r="L23" s="60">
+      <c r="N23" s="60">
         <f>IF(J23="","",J23-F23)</f>
         <v/>
       </c>
-      <c r="M23" s="56" t="n"/>
-      <c r="N23" s="56" t="n"/>
+      <c r="O23" s="56" t="n"/>
+      <c r="P23" s="56" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="47">
       <c r="A24" s="54" t="n"/>
@@ -1804,18 +1889,20 @@
       <c r="E24" s="59" t="n"/>
       <c r="F24" s="60" t="n"/>
       <c r="G24" s="54" t="n"/>
-      <c r="I24" s="61" t="n"/>
-      <c r="J24" s="62" t="n"/>
-      <c r="K24" s="59">
+      <c r="I24" s="92" t="n"/>
+      <c r="J24" s="93" t="n"/>
+      <c r="K24" s="61" t="n"/>
+      <c r="L24" s="62" t="n"/>
+      <c r="M24" s="59">
         <f>IF(I24="","",ROUND(I24-E24,2))</f>
         <v/>
       </c>
-      <c r="L24" s="60">
+      <c r="N24" s="60">
         <f>IF(J24="","",J24-F24)</f>
         <v/>
       </c>
-      <c r="M24" s="56" t="n"/>
-      <c r="N24" s="56" t="n"/>
+      <c r="O24" s="56" t="n"/>
+      <c r="P24" s="56" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="47">
       <c r="A25" s="54" t="n"/>
@@ -1825,18 +1912,20 @@
       <c r="E25" s="59" t="n"/>
       <c r="F25" s="60" t="n"/>
       <c r="G25" s="54" t="n"/>
-      <c r="I25" s="61" t="n"/>
-      <c r="J25" s="62" t="n"/>
-      <c r="K25" s="59">
+      <c r="I25" s="92" t="n"/>
+      <c r="J25" s="93" t="n"/>
+      <c r="K25" s="61" t="n"/>
+      <c r="L25" s="62" t="n"/>
+      <c r="M25" s="59">
         <f>IF(I25="","",ROUND(I25-E25,2))</f>
         <v/>
       </c>
-      <c r="L25" s="60">
+      <c r="N25" s="60">
         <f>IF(J25="","",J25-F25)</f>
         <v/>
       </c>
-      <c r="M25" s="56" t="n"/>
-      <c r="N25" s="56" t="n"/>
+      <c r="O25" s="56" t="n"/>
+      <c r="P25" s="56" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="47">
       <c r="A26" s="54" t="n"/>
@@ -1846,18 +1935,20 @@
       <c r="E26" s="59" t="n"/>
       <c r="F26" s="60" t="n"/>
       <c r="G26" s="54" t="n"/>
-      <c r="I26" s="61" t="n"/>
-      <c r="J26" s="62" t="n"/>
-      <c r="K26" s="59">
+      <c r="I26" s="92" t="n"/>
+      <c r="J26" s="93" t="n"/>
+      <c r="K26" s="61" t="n"/>
+      <c r="L26" s="62" t="n"/>
+      <c r="M26" s="59">
         <f>IF(I26="","",ROUND(I26-E26,2))</f>
         <v/>
       </c>
-      <c r="L26" s="60">
+      <c r="N26" s="60">
         <f>IF(J26="","",J26-F26)</f>
         <v/>
       </c>
-      <c r="M26" s="56" t="n"/>
-      <c r="N26" s="56" t="n"/>
+      <c r="O26" s="56" t="n"/>
+      <c r="P26" s="56" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="47">
       <c r="A27" s="54" t="n"/>
@@ -1867,18 +1958,20 @@
       <c r="E27" s="59" t="n"/>
       <c r="F27" s="60" t="n"/>
       <c r="G27" s="54" t="n"/>
-      <c r="I27" s="61" t="n"/>
-      <c r="J27" s="62" t="n"/>
-      <c r="K27" s="59">
+      <c r="I27" s="92" t="n"/>
+      <c r="J27" s="93" t="n"/>
+      <c r="K27" s="61" t="n"/>
+      <c r="L27" s="62" t="n"/>
+      <c r="M27" s="59">
         <f>IF(I27="","",ROUND(I27-E27,2))</f>
         <v/>
       </c>
-      <c r="L27" s="60">
+      <c r="N27" s="60">
         <f>IF(J27="","",J27-F27)</f>
         <v/>
       </c>
-      <c r="M27" s="56" t="n"/>
-      <c r="N27" s="56" t="n"/>
+      <c r="O27" s="56" t="n"/>
+      <c r="P27" s="56" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="47">
       <c r="A28" s="54" t="n"/>
@@ -1888,18 +1981,20 @@
       <c r="E28" s="59" t="n"/>
       <c r="F28" s="60" t="n"/>
       <c r="G28" s="54" t="n"/>
-      <c r="I28" s="61" t="n"/>
-      <c r="J28" s="62" t="n"/>
-      <c r="K28" s="59">
+      <c r="I28" s="92" t="n"/>
+      <c r="J28" s="93" t="n"/>
+      <c r="K28" s="61" t="n"/>
+      <c r="L28" s="62" t="n"/>
+      <c r="M28" s="59">
         <f>IF(I28="","",ROUND(I28-E28,2))</f>
         <v/>
       </c>
-      <c r="L28" s="60">
+      <c r="N28" s="60">
         <f>IF(J28="","",J28-F28)</f>
         <v/>
       </c>
-      <c r="M28" s="56" t="n"/>
-      <c r="N28" s="56" t="n"/>
+      <c r="O28" s="56" t="n"/>
+      <c r="P28" s="56" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="47">
       <c r="A29" s="54" t="n"/>
@@ -1909,18 +2004,20 @@
       <c r="E29" s="59" t="n"/>
       <c r="F29" s="60" t="n"/>
       <c r="G29" s="54" t="n"/>
-      <c r="I29" s="61" t="n"/>
-      <c r="J29" s="62" t="n"/>
-      <c r="K29" s="59">
+      <c r="I29" s="92" t="n"/>
+      <c r="J29" s="93" t="n"/>
+      <c r="K29" s="61" t="n"/>
+      <c r="L29" s="62" t="n"/>
+      <c r="M29" s="59">
         <f>IF(I29="","",ROUND(I29-E29,2))</f>
         <v/>
       </c>
-      <c r="L29" s="60">
+      <c r="N29" s="60">
         <f>IF(J29="","",J29-F29)</f>
         <v/>
       </c>
-      <c r="M29" s="56" t="n"/>
-      <c r="N29" s="56" t="n"/>
+      <c r="O29" s="56" t="n"/>
+      <c r="P29" s="56" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="47">
       <c r="A30" s="54" t="n"/>
@@ -1930,18 +2027,20 @@
       <c r="E30" s="59" t="n"/>
       <c r="F30" s="60" t="n"/>
       <c r="G30" s="54" t="n"/>
-      <c r="I30" s="61" t="n"/>
-      <c r="J30" s="62" t="n"/>
-      <c r="K30" s="59">
+      <c r="I30" s="92" t="n"/>
+      <c r="J30" s="93" t="n"/>
+      <c r="K30" s="61" t="n"/>
+      <c r="L30" s="62" t="n"/>
+      <c r="M30" s="59">
         <f>IF(I30="","",ROUND(I30-E30,2))</f>
         <v/>
       </c>
-      <c r="L30" s="60">
+      <c r="N30" s="60">
         <f>IF(J30="","",J30-F30)</f>
         <v/>
       </c>
-      <c r="M30" s="56" t="n"/>
-      <c r="N30" s="56" t="n"/>
+      <c r="O30" s="56" t="n"/>
+      <c r="P30" s="56" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="47">
       <c r="A31" s="54" t="n"/>
@@ -1951,18 +2050,20 @@
       <c r="E31" s="59" t="n"/>
       <c r="F31" s="60" t="n"/>
       <c r="G31" s="54" t="n"/>
-      <c r="I31" s="61" t="n"/>
-      <c r="J31" s="62" t="n"/>
-      <c r="K31" s="59">
+      <c r="I31" s="92" t="n"/>
+      <c r="J31" s="93" t="n"/>
+      <c r="K31" s="61" t="n"/>
+      <c r="L31" s="62" t="n"/>
+      <c r="M31" s="59">
         <f>IF(I31="","",ROUND(I31-E31,2))</f>
         <v/>
       </c>
-      <c r="L31" s="60">
+      <c r="N31" s="60">
         <f>IF(J31="","",J31-F31)</f>
         <v/>
       </c>
-      <c r="M31" s="56" t="n"/>
-      <c r="N31" s="56" t="n"/>
+      <c r="O31" s="56" t="n"/>
+      <c r="P31" s="56" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="47">
       <c r="A32" s="54" t="n"/>
@@ -1972,18 +2073,20 @@
       <c r="E32" s="59" t="n"/>
       <c r="F32" s="60" t="n"/>
       <c r="G32" s="54" t="n"/>
-      <c r="I32" s="61" t="n"/>
-      <c r="J32" s="62" t="n"/>
-      <c r="K32" s="59">
+      <c r="I32" s="92" t="n"/>
+      <c r="J32" s="93" t="n"/>
+      <c r="K32" s="61" t="n"/>
+      <c r="L32" s="62" t="n"/>
+      <c r="M32" s="59">
         <f>IF(I32="","",ROUND(I32-E32,2))</f>
         <v/>
       </c>
-      <c r="L32" s="60">
+      <c r="N32" s="60">
         <f>IF(J32="","",J32-F32)</f>
         <v/>
       </c>
-      <c r="M32" s="56" t="n"/>
-      <c r="N32" s="56" t="n"/>
+      <c r="O32" s="56" t="n"/>
+      <c r="P32" s="56" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="47">
       <c r="A33" s="54" t="n"/>
@@ -1993,18 +2096,20 @@
       <c r="E33" s="59" t="n"/>
       <c r="F33" s="60" t="n"/>
       <c r="G33" s="54" t="n"/>
-      <c r="I33" s="61" t="n"/>
-      <c r="J33" s="62" t="n"/>
-      <c r="K33" s="59">
+      <c r="I33" s="92" t="n"/>
+      <c r="J33" s="93" t="n"/>
+      <c r="K33" s="61" t="n"/>
+      <c r="L33" s="62" t="n"/>
+      <c r="M33" s="59">
         <f>IF(I33="","",ROUND(I33-E33,2))</f>
         <v/>
       </c>
-      <c r="L33" s="60">
+      <c r="N33" s="60">
         <f>IF(J33="","",J33-F33)</f>
         <v/>
       </c>
-      <c r="M33" s="56" t="n"/>
-      <c r="N33" s="56" t="n"/>
+      <c r="O33" s="56" t="n"/>
+      <c r="P33" s="56" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="47">
       <c r="A34" s="54" t="n"/>
@@ -2014,18 +2119,20 @@
       <c r="E34" s="59" t="n"/>
       <c r="F34" s="60" t="n"/>
       <c r="G34" s="54" t="n"/>
-      <c r="I34" s="61" t="n"/>
-      <c r="J34" s="62" t="n"/>
-      <c r="K34" s="59">
+      <c r="I34" s="92" t="n"/>
+      <c r="J34" s="93" t="n"/>
+      <c r="K34" s="61" t="n"/>
+      <c r="L34" s="62" t="n"/>
+      <c r="M34" s="59">
         <f>IF(I34="","",ROUND(I34-E34,2))</f>
         <v/>
       </c>
-      <c r="L34" s="60">
+      <c r="N34" s="60">
         <f>IF(J34="","",J34-F34)</f>
         <v/>
       </c>
-      <c r="M34" s="56" t="n"/>
-      <c r="N34" s="56" t="n"/>
+      <c r="O34" s="56" t="n"/>
+      <c r="P34" s="56" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="47">
       <c r="A35" s="54" t="n"/>
@@ -2035,18 +2142,20 @@
       <c r="E35" s="59" t="n"/>
       <c r="F35" s="60" t="n"/>
       <c r="G35" s="54" t="n"/>
-      <c r="I35" s="61" t="n"/>
-      <c r="J35" s="62" t="n"/>
-      <c r="K35" s="59">
+      <c r="I35" s="92" t="n"/>
+      <c r="J35" s="93" t="n"/>
+      <c r="K35" s="61" t="n"/>
+      <c r="L35" s="62" t="n"/>
+      <c r="M35" s="59">
         <f>IF(I35="","",ROUND(I35-E35,2))</f>
         <v/>
       </c>
-      <c r="L35" s="60">
+      <c r="N35" s="60">
         <f>IF(J35="","",J35-F35)</f>
         <v/>
       </c>
-      <c r="M35" s="56" t="n"/>
-      <c r="N35" s="56" t="n"/>
+      <c r="O35" s="56" t="n"/>
+      <c r="P35" s="56" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="47">
       <c r="A36" s="54" t="n"/>
@@ -2056,18 +2165,20 @@
       <c r="E36" s="59" t="n"/>
       <c r="F36" s="60" t="n"/>
       <c r="G36" s="54" t="n"/>
-      <c r="I36" s="61" t="n"/>
-      <c r="J36" s="62" t="n"/>
-      <c r="K36" s="59">
+      <c r="I36" s="92" t="n"/>
+      <c r="J36" s="93" t="n"/>
+      <c r="K36" s="61" t="n"/>
+      <c r="L36" s="62" t="n"/>
+      <c r="M36" s="59">
         <f>IF(I36="","",ROUND(I36-E36,2))</f>
         <v/>
       </c>
-      <c r="L36" s="60">
+      <c r="N36" s="60">
         <f>IF(J36="","",J36-F36)</f>
         <v/>
       </c>
-      <c r="M36" s="56" t="n"/>
-      <c r="N36" s="56" t="n"/>
+      <c r="O36" s="56" t="n"/>
+      <c r="P36" s="56" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="47">
       <c r="A37" s="54" t="n"/>
@@ -2077,18 +2188,20 @@
       <c r="E37" s="59" t="n"/>
       <c r="F37" s="60" t="n"/>
       <c r="G37" s="54" t="n"/>
-      <c r="I37" s="61" t="n"/>
-      <c r="J37" s="62" t="n"/>
-      <c r="K37" s="59">
+      <c r="I37" s="92" t="n"/>
+      <c r="J37" s="93" t="n"/>
+      <c r="K37" s="61" t="n"/>
+      <c r="L37" s="62" t="n"/>
+      <c r="M37" s="59">
         <f>IF(I37="","",ROUND(I37-E37,2))</f>
         <v/>
       </c>
-      <c r="L37" s="60">
+      <c r="N37" s="60">
         <f>IF(J37="","",J37-F37)</f>
         <v/>
       </c>
-      <c r="M37" s="56" t="n"/>
-      <c r="N37" s="56" t="n"/>
+      <c r="O37" s="56" t="n"/>
+      <c r="P37" s="56" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="47">
       <c r="A38" s="54" t="n"/>
@@ -2098,18 +2211,20 @@
       <c r="E38" s="59" t="n"/>
       <c r="F38" s="60" t="n"/>
       <c r="G38" s="54" t="n"/>
-      <c r="I38" s="61" t="n"/>
-      <c r="J38" s="62" t="n"/>
-      <c r="K38" s="59">
+      <c r="I38" s="92" t="n"/>
+      <c r="J38" s="93" t="n"/>
+      <c r="K38" s="61" t="n"/>
+      <c r="L38" s="62" t="n"/>
+      <c r="M38" s="59">
         <f>IF(I38="","",ROUND(I38-E38,2))</f>
         <v/>
       </c>
-      <c r="L38" s="60">
+      <c r="N38" s="60">
         <f>IF(J38="","",J38-F38)</f>
         <v/>
       </c>
-      <c r="M38" s="56" t="n"/>
-      <c r="N38" s="56" t="n"/>
+      <c r="O38" s="56" t="n"/>
+      <c r="P38" s="56" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="47">
       <c r="A39" s="54" t="n"/>
@@ -2119,18 +2234,20 @@
       <c r="E39" s="59" t="n"/>
       <c r="F39" s="60" t="n"/>
       <c r="G39" s="54" t="n"/>
-      <c r="I39" s="61" t="n"/>
-      <c r="J39" s="62" t="n"/>
-      <c r="K39" s="59">
+      <c r="I39" s="92" t="n"/>
+      <c r="J39" s="93" t="n"/>
+      <c r="K39" s="61" t="n"/>
+      <c r="L39" s="62" t="n"/>
+      <c r="M39" s="59">
         <f>IF(I39="","",ROUND(I39-E39,2))</f>
         <v/>
       </c>
-      <c r="L39" s="60">
+      <c r="N39" s="60">
         <f>IF(J39="","",J39-F39)</f>
         <v/>
       </c>
-      <c r="M39" s="56" t="n"/>
-      <c r="N39" s="56" t="n"/>
+      <c r="O39" s="56" t="n"/>
+      <c r="P39" s="56" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="47">
       <c r="A40" s="54" t="n"/>
@@ -2140,18 +2257,20 @@
       <c r="E40" s="59" t="n"/>
       <c r="F40" s="60" t="n"/>
       <c r="G40" s="54" t="n"/>
-      <c r="I40" s="61" t="n"/>
-      <c r="J40" s="62" t="n"/>
-      <c r="K40" s="59">
+      <c r="I40" s="92" t="n"/>
+      <c r="J40" s="93" t="n"/>
+      <c r="K40" s="61" t="n"/>
+      <c r="L40" s="62" t="n"/>
+      <c r="M40" s="59">
         <f>IF(I40="","",ROUND(I40-E40,2))</f>
         <v/>
       </c>
-      <c r="L40" s="60">
+      <c r="N40" s="60">
         <f>IF(J40="","",J40-F40)</f>
         <v/>
       </c>
-      <c r="M40" s="56" t="n"/>
-      <c r="N40" s="56" t="n"/>
+      <c r="O40" s="56" t="n"/>
+      <c r="P40" s="56" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="47">
       <c r="A41" s="54" t="n"/>
@@ -2161,18 +2280,20 @@
       <c r="E41" s="59" t="n"/>
       <c r="F41" s="60" t="n"/>
       <c r="G41" s="54" t="n"/>
-      <c r="I41" s="61" t="n"/>
-      <c r="J41" s="62" t="n"/>
-      <c r="K41" s="59">
+      <c r="I41" s="92" t="n"/>
+      <c r="J41" s="93" t="n"/>
+      <c r="K41" s="61" t="n"/>
+      <c r="L41" s="62" t="n"/>
+      <c r="M41" s="59">
         <f>IF(I41="","",ROUND(I41-E41,2))</f>
         <v/>
       </c>
-      <c r="L41" s="60">
+      <c r="N41" s="60">
         <f>IF(J41="","",J41-F41)</f>
         <v/>
       </c>
-      <c r="M41" s="56" t="n"/>
-      <c r="N41" s="56" t="n"/>
+      <c r="O41" s="56" t="n"/>
+      <c r="P41" s="56" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="47">
       <c r="A42" s="54" t="n"/>
@@ -2182,18 +2303,20 @@
       <c r="E42" s="59" t="n"/>
       <c r="F42" s="60" t="n"/>
       <c r="G42" s="54" t="n"/>
-      <c r="I42" s="61" t="n"/>
-      <c r="J42" s="62" t="n"/>
-      <c r="K42" s="59">
+      <c r="I42" s="92" t="n"/>
+      <c r="J42" s="93" t="n"/>
+      <c r="K42" s="61" t="n"/>
+      <c r="L42" s="62" t="n"/>
+      <c r="M42" s="59">
         <f>IF(I42="","",ROUND(I42-E42,2))</f>
         <v/>
       </c>
-      <c r="L42" s="60">
+      <c r="N42" s="60">
         <f>IF(J42="","",J42-F42)</f>
         <v/>
       </c>
-      <c r="M42" s="56" t="n"/>
-      <c r="N42" s="56" t="n"/>
+      <c r="O42" s="56" t="n"/>
+      <c r="P42" s="56" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="47">
       <c r="A43" s="54" t="n"/>
@@ -2203,18 +2326,20 @@
       <c r="E43" s="59" t="n"/>
       <c r="F43" s="60" t="n"/>
       <c r="G43" s="54" t="n"/>
-      <c r="I43" s="61" t="n"/>
-      <c r="J43" s="62" t="n"/>
-      <c r="K43" s="59">
+      <c r="I43" s="92" t="n"/>
+      <c r="J43" s="93" t="n"/>
+      <c r="K43" s="61" t="n"/>
+      <c r="L43" s="62" t="n"/>
+      <c r="M43" s="59">
         <f>IF(I43="","",ROUND(I43-E43,2))</f>
         <v/>
       </c>
-      <c r="L43" s="60">
+      <c r="N43" s="60">
         <f>IF(J43="","",J43-F43)</f>
         <v/>
       </c>
-      <c r="M43" s="56" t="n"/>
-      <c r="N43" s="56" t="n"/>
+      <c r="O43" s="56" t="n"/>
+      <c r="P43" s="56" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="47">
       <c r="A44" s="54" t="n"/>
@@ -2224,18 +2349,20 @@
       <c r="E44" s="59" t="n"/>
       <c r="F44" s="60" t="n"/>
       <c r="G44" s="54" t="n"/>
-      <c r="I44" s="61" t="n"/>
-      <c r="J44" s="62" t="n"/>
-      <c r="K44" s="59">
+      <c r="I44" s="92" t="n"/>
+      <c r="J44" s="93" t="n"/>
+      <c r="K44" s="61" t="n"/>
+      <c r="L44" s="62" t="n"/>
+      <c r="M44" s="59">
         <f>IF(I44="","",ROUND(I44-E44,2))</f>
         <v/>
       </c>
-      <c r="L44" s="60">
+      <c r="N44" s="60">
         <f>IF(J44="","",J44-F44)</f>
         <v/>
       </c>
-      <c r="M44" s="56" t="n"/>
-      <c r="N44" s="56" t="n"/>
+      <c r="O44" s="56" t="n"/>
+      <c r="P44" s="56" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="47">
       <c r="A45" s="54" t="n"/>
@@ -2245,18 +2372,20 @@
       <c r="E45" s="59" t="n"/>
       <c r="F45" s="60" t="n"/>
       <c r="G45" s="54" t="n"/>
-      <c r="I45" s="61" t="n"/>
-      <c r="J45" s="62" t="n"/>
-      <c r="K45" s="59">
+      <c r="I45" s="92" t="n"/>
+      <c r="J45" s="93" t="n"/>
+      <c r="K45" s="61" t="n"/>
+      <c r="L45" s="62" t="n"/>
+      <c r="M45" s="59">
         <f>IF(I45="","",ROUND(I45-E45,2))</f>
         <v/>
       </c>
-      <c r="L45" s="60">
+      <c r="N45" s="60">
         <f>IF(J45="","",J45-F45)</f>
         <v/>
       </c>
-      <c r="M45" s="56" t="n"/>
-      <c r="N45" s="56" t="n"/>
+      <c r="O45" s="56" t="n"/>
+      <c r="P45" s="56" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="47">
       <c r="A46" s="54" t="n"/>
@@ -2266,18 +2395,20 @@
       <c r="E46" s="59" t="n"/>
       <c r="F46" s="60" t="n"/>
       <c r="G46" s="54" t="n"/>
-      <c r="I46" s="61" t="n"/>
-      <c r="J46" s="62" t="n"/>
-      <c r="K46" s="59">
+      <c r="I46" s="92" t="n"/>
+      <c r="J46" s="93" t="n"/>
+      <c r="K46" s="61" t="n"/>
+      <c r="L46" s="62" t="n"/>
+      <c r="M46" s="59">
         <f>IF(I46="","",ROUND(I46-E46,2))</f>
         <v/>
       </c>
-      <c r="L46" s="60">
+      <c r="N46" s="60">
         <f>IF(J46="","",J46-F46)</f>
         <v/>
       </c>
-      <c r="M46" s="56" t="n"/>
-      <c r="N46" s="56" t="n"/>
+      <c r="O46" s="56" t="n"/>
+      <c r="P46" s="56" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="47">
       <c r="A47" s="54" t="n"/>
@@ -2287,18 +2418,20 @@
       <c r="E47" s="59" t="n"/>
       <c r="F47" s="60" t="n"/>
       <c r="G47" s="54" t="n"/>
-      <c r="I47" s="61" t="n"/>
-      <c r="J47" s="62" t="n"/>
-      <c r="K47" s="59">
+      <c r="I47" s="92" t="n"/>
+      <c r="J47" s="93" t="n"/>
+      <c r="K47" s="61" t="n"/>
+      <c r="L47" s="62" t="n"/>
+      <c r="M47" s="59">
         <f>IF(I47="","",ROUND(I47-E47,2))</f>
         <v/>
       </c>
-      <c r="L47" s="60">
+      <c r="N47" s="60">
         <f>IF(J47="","",J47-F47)</f>
         <v/>
       </c>
-      <c r="M47" s="56" t="n"/>
-      <c r="N47" s="56" t="n"/>
+      <c r="O47" s="56" t="n"/>
+      <c r="P47" s="56" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="47">
       <c r="A48" s="54" t="n"/>
@@ -2308,18 +2441,20 @@
       <c r="E48" s="59" t="n"/>
       <c r="F48" s="60" t="n"/>
       <c r="G48" s="54" t="n"/>
-      <c r="I48" s="61" t="n"/>
-      <c r="J48" s="62" t="n"/>
-      <c r="K48" s="59">
+      <c r="I48" s="92" t="n"/>
+      <c r="J48" s="93" t="n"/>
+      <c r="K48" s="61" t="n"/>
+      <c r="L48" s="62" t="n"/>
+      <c r="M48" s="59">
         <f>IF(I48="","",ROUND(I48-E48,2))</f>
         <v/>
       </c>
-      <c r="L48" s="60">
+      <c r="N48" s="60">
         <f>IF(J48="","",J48-F48)</f>
         <v/>
       </c>
-      <c r="M48" s="56" t="n"/>
-      <c r="N48" s="56" t="n"/>
+      <c r="O48" s="56" t="n"/>
+      <c r="P48" s="56" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="47">
       <c r="A49" s="54" t="n"/>
@@ -2329,18 +2464,20 @@
       <c r="E49" s="59" t="n"/>
       <c r="F49" s="60" t="n"/>
       <c r="G49" s="54" t="n"/>
-      <c r="I49" s="61" t="n"/>
-      <c r="J49" s="62" t="n"/>
-      <c r="K49" s="59">
+      <c r="I49" s="92" t="n"/>
+      <c r="J49" s="93" t="n"/>
+      <c r="K49" s="61" t="n"/>
+      <c r="L49" s="62" t="n"/>
+      <c r="M49" s="59">
         <f>IF(I49="","",ROUND(I49-E49,2))</f>
         <v/>
       </c>
-      <c r="L49" s="60">
+      <c r="N49" s="60">
         <f>IF(J49="","",J49-F49)</f>
         <v/>
       </c>
-      <c r="M49" s="56" t="n"/>
-      <c r="N49" s="56" t="n"/>
+      <c r="O49" s="56" t="n"/>
+      <c r="P49" s="56" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="47">
       <c r="A50" s="54" t="n"/>
@@ -2350,18 +2487,20 @@
       <c r="E50" s="59" t="n"/>
       <c r="F50" s="60" t="n"/>
       <c r="G50" s="54" t="n"/>
-      <c r="I50" s="61" t="n"/>
-      <c r="J50" s="62" t="n"/>
-      <c r="K50" s="59">
+      <c r="I50" s="92" t="n"/>
+      <c r="J50" s="93" t="n"/>
+      <c r="K50" s="61" t="n"/>
+      <c r="L50" s="62" t="n"/>
+      <c r="M50" s="59">
         <f>IF(I50="","",ROUND(I50-E50,2))</f>
         <v/>
       </c>
-      <c r="L50" s="60">
+      <c r="N50" s="60">
         <f>IF(J50="","",J50-F50)</f>
         <v/>
       </c>
-      <c r="M50" s="56" t="n"/>
-      <c r="N50" s="56" t="inlineStr">
+      <c r="O50" s="56" t="n"/>
+      <c r="P50" s="56" t="inlineStr">
         <is>
           <t>Check reception date — dated in the future in the app</t>
         </is>
@@ -2375,18 +2514,20 @@
       <c r="E51" s="59" t="n"/>
       <c r="F51" s="60" t="n"/>
       <c r="G51" s="54" t="n"/>
-      <c r="I51" s="61" t="n"/>
-      <c r="J51" s="62" t="n"/>
-      <c r="K51" s="59">
+      <c r="I51" s="92" t="n"/>
+      <c r="J51" s="93" t="n"/>
+      <c r="K51" s="61" t="n"/>
+      <c r="L51" s="62" t="n"/>
+      <c r="M51" s="59">
         <f>IF(I51="","",ROUND(I51-E51,2))</f>
         <v/>
       </c>
-      <c r="L51" s="60">
+      <c r="N51" s="60">
         <f>IF(J51="","",J51-F51)</f>
         <v/>
       </c>
-      <c r="M51" s="56" t="n"/>
-      <c r="N51" s="56" t="n"/>
+      <c r="O51" s="56" t="n"/>
+      <c r="P51" s="56" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="47">
       <c r="A52" s="54" t="n"/>
@@ -2396,18 +2537,20 @@
       <c r="E52" s="59" t="n"/>
       <c r="F52" s="60" t="n"/>
       <c r="G52" s="54" t="n"/>
-      <c r="I52" s="61" t="n"/>
-      <c r="J52" s="62" t="n"/>
-      <c r="K52" s="59">
+      <c r="I52" s="92" t="n"/>
+      <c r="J52" s="93" t="n"/>
+      <c r="K52" s="61" t="n"/>
+      <c r="L52" s="62" t="n"/>
+      <c r="M52" s="59">
         <f>IF(I52="","",ROUND(I52-E52,2))</f>
         <v/>
       </c>
-      <c r="L52" s="60">
+      <c r="N52" s="60">
         <f>IF(J52="","",J52-F52)</f>
         <v/>
       </c>
-      <c r="M52" s="56" t="n"/>
-      <c r="N52" s="56" t="n"/>
+      <c r="O52" s="56" t="n"/>
+      <c r="P52" s="56" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="47">
       <c r="A53" s="54" t="n"/>
@@ -2417,18 +2560,20 @@
       <c r="E53" s="59" t="n"/>
       <c r="F53" s="60" t="n"/>
       <c r="G53" s="54" t="n"/>
-      <c r="I53" s="61" t="n"/>
-      <c r="J53" s="62" t="n"/>
-      <c r="K53" s="59">
+      <c r="I53" s="92" t="n"/>
+      <c r="J53" s="93" t="n"/>
+      <c r="K53" s="61" t="n"/>
+      <c r="L53" s="62" t="n"/>
+      <c r="M53" s="59">
         <f>IF(I53="","",ROUND(I53-E53,2))</f>
         <v/>
       </c>
-      <c r="L53" s="60">
+      <c r="N53" s="60">
         <f>IF(J53="","",J53-F53)</f>
         <v/>
       </c>
-      <c r="M53" s="56" t="n"/>
-      <c r="N53" s="56" t="n"/>
+      <c r="O53" s="56" t="n"/>
+      <c r="P53" s="56" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="47">
       <c r="A54" s="54" t="n"/>
@@ -2438,18 +2583,20 @@
       <c r="E54" s="59" t="n"/>
       <c r="F54" s="60" t="n"/>
       <c r="G54" s="54" t="n"/>
-      <c r="I54" s="61" t="n"/>
-      <c r="J54" s="62" t="n"/>
-      <c r="K54" s="59">
+      <c r="I54" s="92" t="n"/>
+      <c r="J54" s="93" t="n"/>
+      <c r="K54" s="61" t="n"/>
+      <c r="L54" s="62" t="n"/>
+      <c r="M54" s="59">
         <f>IF(I54="","",ROUND(I54-E54,2))</f>
         <v/>
       </c>
-      <c r="L54" s="60">
+      <c r="N54" s="60">
         <f>IF(J54="","",J54-F54)</f>
         <v/>
       </c>
-      <c r="M54" s="56" t="n"/>
-      <c r="N54" s="56" t="n"/>
+      <c r="O54" s="56" t="n"/>
+      <c r="P54" s="56" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="47">
       <c r="A55" s="54" t="n"/>
@@ -2459,18 +2606,20 @@
       <c r="E55" s="59" t="n"/>
       <c r="F55" s="60" t="n"/>
       <c r="G55" s="54" t="n"/>
-      <c r="I55" s="61" t="n"/>
-      <c r="J55" s="62" t="n"/>
-      <c r="K55" s="59">
+      <c r="I55" s="92" t="n"/>
+      <c r="J55" s="93" t="n"/>
+      <c r="K55" s="61" t="n"/>
+      <c r="L55" s="62" t="n"/>
+      <c r="M55" s="59">
         <f>IF(I55="","",ROUND(I55-E55,2))</f>
         <v/>
       </c>
-      <c r="L55" s="60">
+      <c r="N55" s="60">
         <f>IF(J55="","",J55-F55)</f>
         <v/>
       </c>
-      <c r="M55" s="56" t="n"/>
-      <c r="N55" s="56" t="n"/>
+      <c r="O55" s="56" t="n"/>
+      <c r="P55" s="56" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="47">
       <c r="A56" s="54" t="n"/>
@@ -2480,18 +2629,20 @@
       <c r="E56" s="59" t="n"/>
       <c r="F56" s="60" t="n"/>
       <c r="G56" s="54" t="n"/>
-      <c r="I56" s="61" t="n"/>
-      <c r="J56" s="62" t="n"/>
-      <c r="K56" s="59">
+      <c r="I56" s="92" t="n"/>
+      <c r="J56" s="93" t="n"/>
+      <c r="K56" s="61" t="n"/>
+      <c r="L56" s="62" t="n"/>
+      <c r="M56" s="59">
         <f>IF(I56="","",ROUND(I56-E56,2))</f>
         <v/>
       </c>
-      <c r="L56" s="60">
+      <c r="N56" s="60">
         <f>IF(J56="","",J56-F56)</f>
         <v/>
       </c>
-      <c r="M56" s="56" t="n"/>
-      <c r="N56" s="56" t="n"/>
+      <c r="O56" s="56" t="n"/>
+      <c r="P56" s="56" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="47">
       <c r="A57" s="54" t="n"/>
@@ -2501,18 +2652,20 @@
       <c r="E57" s="59" t="n"/>
       <c r="F57" s="60" t="n"/>
       <c r="G57" s="54" t="n"/>
-      <c r="I57" s="61" t="n"/>
-      <c r="J57" s="62" t="n"/>
-      <c r="K57" s="59">
+      <c r="I57" s="92" t="n"/>
+      <c r="J57" s="93" t="n"/>
+      <c r="K57" s="61" t="n"/>
+      <c r="L57" s="62" t="n"/>
+      <c r="M57" s="59">
         <f>IF(I57="","",ROUND(I57-E57,2))</f>
         <v/>
       </c>
-      <c r="L57" s="60">
+      <c r="N57" s="60">
         <f>IF(J57="","",J57-F57)</f>
         <v/>
       </c>
-      <c r="M57" s="56" t="n"/>
-      <c r="N57" s="56" t="n"/>
+      <c r="O57" s="56" t="n"/>
+      <c r="P57" s="56" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="47">
       <c r="A58" s="54" t="n"/>
@@ -2522,18 +2675,20 @@
       <c r="E58" s="59" t="n"/>
       <c r="F58" s="60" t="n"/>
       <c r="G58" s="54" t="n"/>
-      <c r="I58" s="61" t="n"/>
-      <c r="J58" s="62" t="n"/>
-      <c r="K58" s="59">
+      <c r="I58" s="92" t="n"/>
+      <c r="J58" s="93" t="n"/>
+      <c r="K58" s="61" t="n"/>
+      <c r="L58" s="62" t="n"/>
+      <c r="M58" s="59">
         <f>IF(I58="","",ROUND(I58-E58,2))</f>
         <v/>
       </c>
-      <c r="L58" s="60">
+      <c r="N58" s="60">
         <f>IF(J58="","",J58-F58)</f>
         <v/>
       </c>
-      <c r="M58" s="56" t="n"/>
-      <c r="N58" s="56" t="n"/>
+      <c r="O58" s="56" t="n"/>
+      <c r="P58" s="56" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="47">
       <c r="A59" s="54" t="n"/>
@@ -2543,18 +2698,20 @@
       <c r="E59" s="59" t="n"/>
       <c r="F59" s="60" t="n"/>
       <c r="G59" s="54" t="n"/>
-      <c r="I59" s="61" t="n"/>
-      <c r="J59" s="62" t="n"/>
-      <c r="K59" s="59">
+      <c r="I59" s="92" t="n"/>
+      <c r="J59" s="93" t="n"/>
+      <c r="K59" s="61" t="n"/>
+      <c r="L59" s="62" t="n"/>
+      <c r="M59" s="59">
         <f>IF(I59="","",ROUND(I59-E59,2))</f>
         <v/>
       </c>
-      <c r="L59" s="60">
+      <c r="N59" s="60">
         <f>IF(J59="","",J59-F59)</f>
         <v/>
       </c>
-      <c r="M59" s="56" t="n"/>
-      <c r="N59" s="56" t="n"/>
+      <c r="O59" s="56" t="n"/>
+      <c r="P59" s="56" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="47">
       <c r="A60" s="54" t="n"/>
@@ -2564,18 +2721,20 @@
       <c r="E60" s="59" t="n"/>
       <c r="F60" s="60" t="n"/>
       <c r="G60" s="54" t="n"/>
-      <c r="I60" s="61" t="n"/>
-      <c r="J60" s="62" t="n"/>
-      <c r="K60" s="59">
+      <c r="I60" s="92" t="n"/>
+      <c r="J60" s="93" t="n"/>
+      <c r="K60" s="61" t="n"/>
+      <c r="L60" s="62" t="n"/>
+      <c r="M60" s="59">
         <f>IF(I60="","",ROUND(I60-E60,2))</f>
         <v/>
       </c>
-      <c r="L60" s="60">
+      <c r="N60" s="60">
         <f>IF(J60="","",J60-F60)</f>
         <v/>
       </c>
-      <c r="M60" s="56" t="n"/>
-      <c r="N60" s="56" t="n"/>
+      <c r="O60" s="56" t="n"/>
+      <c r="P60" s="56" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="47">
       <c r="A61" s="54" t="n"/>
@@ -2585,18 +2744,20 @@
       <c r="E61" s="59" t="n"/>
       <c r="F61" s="60" t="n"/>
       <c r="G61" s="54" t="n"/>
-      <c r="I61" s="61" t="n"/>
-      <c r="J61" s="62" t="n"/>
-      <c r="K61" s="59">
+      <c r="I61" s="92" t="n"/>
+      <c r="J61" s="93" t="n"/>
+      <c r="K61" s="61" t="n"/>
+      <c r="L61" s="62" t="n"/>
+      <c r="M61" s="59">
         <f>IF(I61="","",ROUND(I61-E61,2))</f>
         <v/>
       </c>
-      <c r="L61" s="60">
+      <c r="N61" s="60">
         <f>IF(J61="","",J61-F61)</f>
         <v/>
       </c>
-      <c r="M61" s="56" t="n"/>
-      <c r="N61" s="56" t="n"/>
+      <c r="O61" s="56" t="n"/>
+      <c r="P61" s="56" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="47">
       <c r="A62" s="54" t="n"/>
@@ -2606,18 +2767,20 @@
       <c r="E62" s="59" t="n"/>
       <c r="F62" s="60" t="n"/>
       <c r="G62" s="54" t="n"/>
-      <c r="I62" s="61" t="n"/>
-      <c r="J62" s="62" t="n"/>
-      <c r="K62" s="59">
+      <c r="I62" s="92" t="n"/>
+      <c r="J62" s="93" t="n"/>
+      <c r="K62" s="61" t="n"/>
+      <c r="L62" s="62" t="n"/>
+      <c r="M62" s="59">
         <f>IF(I62="","",ROUND(I62-E62,2))</f>
         <v/>
       </c>
-      <c r="L62" s="60">
+      <c r="N62" s="60">
         <f>IF(J62="","",J62-F62)</f>
         <v/>
       </c>
-      <c r="M62" s="56" t="n"/>
-      <c r="N62" s="56" t="n"/>
+      <c r="O62" s="56" t="n"/>
+      <c r="P62" s="56" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="47">
       <c r="A63" s="54" t="n"/>
@@ -2627,18 +2790,20 @@
       <c r="E63" s="59" t="n"/>
       <c r="F63" s="60" t="n"/>
       <c r="G63" s="54" t="n"/>
-      <c r="I63" s="61" t="n"/>
-      <c r="J63" s="62" t="n"/>
-      <c r="K63" s="59">
+      <c r="I63" s="92" t="n"/>
+      <c r="J63" s="93" t="n"/>
+      <c r="K63" s="61" t="n"/>
+      <c r="L63" s="62" t="n"/>
+      <c r="M63" s="59">
         <f>IF(I63="","",ROUND(I63-E63,2))</f>
         <v/>
       </c>
-      <c r="L63" s="60">
+      <c r="N63" s="60">
         <f>IF(J63="","",J63-F63)</f>
         <v/>
       </c>
-      <c r="M63" s="56" t="n"/>
-      <c r="N63" s="56" t="n"/>
+      <c r="O63" s="56" t="n"/>
+      <c r="P63" s="56" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="47">
       <c r="A64" s="54" t="n"/>
@@ -2648,18 +2813,20 @@
       <c r="E64" s="59" t="n"/>
       <c r="F64" s="60" t="n"/>
       <c r="G64" s="54" t="n"/>
-      <c r="I64" s="61" t="n"/>
-      <c r="J64" s="62" t="n"/>
-      <c r="K64" s="59">
+      <c r="I64" s="92" t="n"/>
+      <c r="J64" s="93" t="n"/>
+      <c r="K64" s="61" t="n"/>
+      <c r="L64" s="62" t="n"/>
+      <c r="M64" s="59">
         <f>IF(I64="","",ROUND(I64-E64,2))</f>
         <v/>
       </c>
-      <c r="L64" s="60">
+      <c r="N64" s="60">
         <f>IF(J64="","",J64-F64)</f>
         <v/>
       </c>
-      <c r="M64" s="56" t="n"/>
-      <c r="N64" s="56" t="n"/>
+      <c r="O64" s="56" t="n"/>
+      <c r="P64" s="56" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="47">
       <c r="A65" s="54" t="n"/>
@@ -2669,18 +2836,20 @@
       <c r="E65" s="59" t="n"/>
       <c r="F65" s="60" t="n"/>
       <c r="G65" s="54" t="n"/>
-      <c r="I65" s="61" t="n"/>
-      <c r="J65" s="62" t="n"/>
-      <c r="K65" s="59">
+      <c r="I65" s="92" t="n"/>
+      <c r="J65" s="93" t="n"/>
+      <c r="K65" s="61" t="n"/>
+      <c r="L65" s="62" t="n"/>
+      <c r="M65" s="59">
         <f>IF(I65="","",ROUND(I65-E65,2))</f>
         <v/>
       </c>
-      <c r="L65" s="60">
+      <c r="N65" s="60">
         <f>IF(J65="","",J65-F65)</f>
         <v/>
       </c>
-      <c r="M65" s="56" t="n"/>
-      <c r="N65" s="56" t="n"/>
+      <c r="O65" s="56" t="n"/>
+      <c r="P65" s="56" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="47">
       <c r="A66" s="54" t="n"/>
@@ -2690,18 +2859,20 @@
       <c r="E66" s="59" t="n"/>
       <c r="F66" s="60" t="n"/>
       <c r="G66" s="54" t="n"/>
-      <c r="I66" s="61" t="n"/>
-      <c r="J66" s="62" t="n"/>
-      <c r="K66" s="59">
+      <c r="I66" s="92" t="n"/>
+      <c r="J66" s="93" t="n"/>
+      <c r="K66" s="61" t="n"/>
+      <c r="L66" s="62" t="n"/>
+      <c r="M66" s="59">
         <f>IF(I66="","",ROUND(I66-E66,2))</f>
         <v/>
       </c>
-      <c r="L66" s="60">
+      <c r="N66" s="60">
         <f>IF(J66="","",J66-F66)</f>
         <v/>
       </c>
-      <c r="M66" s="56" t="n"/>
-      <c r="N66" s="56" t="n"/>
+      <c r="O66" s="56" t="n"/>
+      <c r="P66" s="56" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="47">
       <c r="A67" s="54" t="n"/>
@@ -2711,18 +2882,20 @@
       <c r="E67" s="59" t="n"/>
       <c r="F67" s="60" t="n"/>
       <c r="G67" s="54" t="n"/>
-      <c r="I67" s="61" t="n"/>
-      <c r="J67" s="62" t="n"/>
-      <c r="K67" s="59">
+      <c r="I67" s="92" t="n"/>
+      <c r="J67" s="93" t="n"/>
+      <c r="K67" s="61" t="n"/>
+      <c r="L67" s="62" t="n"/>
+      <c r="M67" s="59">
         <f>IF(I67="","",ROUND(I67-E67,2))</f>
         <v/>
       </c>
-      <c r="L67" s="60">
+      <c r="N67" s="60">
         <f>IF(J67="","",J67-F67)</f>
         <v/>
       </c>
-      <c r="M67" s="56" t="n"/>
-      <c r="N67" s="56" t="n"/>
+      <c r="O67" s="56" t="n"/>
+      <c r="P67" s="56" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="47">
       <c r="A68" s="54" t="n"/>
@@ -2732,18 +2905,20 @@
       <c r="E68" s="59" t="n"/>
       <c r="F68" s="60" t="n"/>
       <c r="G68" s="54" t="n"/>
-      <c r="I68" s="61" t="n"/>
-      <c r="J68" s="62" t="n"/>
-      <c r="K68" s="59">
+      <c r="I68" s="92" t="n"/>
+      <c r="J68" s="93" t="n"/>
+      <c r="K68" s="61" t="n"/>
+      <c r="L68" s="62" t="n"/>
+      <c r="M68" s="59">
         <f>IF(I68="","",ROUND(I68-E68,2))</f>
         <v/>
       </c>
-      <c r="L68" s="60">
+      <c r="N68" s="60">
         <f>IF(J68="","",J68-F68)</f>
         <v/>
       </c>
-      <c r="M68" s="56" t="n"/>
-      <c r="N68" s="56" t="n"/>
+      <c r="O68" s="56" t="n"/>
+      <c r="P68" s="56" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="47">
       <c r="A69" s="54" t="n"/>
@@ -2753,18 +2928,20 @@
       <c r="E69" s="59" t="n"/>
       <c r="F69" s="60" t="n"/>
       <c r="G69" s="54" t="n"/>
-      <c r="I69" s="61" t="n"/>
-      <c r="J69" s="62" t="n"/>
-      <c r="K69" s="59">
+      <c r="I69" s="92" t="n"/>
+      <c r="J69" s="93" t="n"/>
+      <c r="K69" s="61" t="n"/>
+      <c r="L69" s="62" t="n"/>
+      <c r="M69" s="59">
         <f>IF(I69="","",ROUND(I69-E69,2))</f>
         <v/>
       </c>
-      <c r="L69" s="60">
+      <c r="N69" s="60">
         <f>IF(J69="","",J69-F69)</f>
         <v/>
       </c>
-      <c r="M69" s="56" t="n"/>
-      <c r="N69" s="56" t="n"/>
+      <c r="O69" s="56" t="n"/>
+      <c r="P69" s="56" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="47">
       <c r="A70" s="54" t="n"/>
@@ -2774,18 +2951,20 @@
       <c r="E70" s="59" t="n"/>
       <c r="F70" s="60" t="n"/>
       <c r="G70" s="54" t="n"/>
-      <c r="I70" s="61" t="n"/>
-      <c r="J70" s="62" t="n"/>
-      <c r="K70" s="59">
+      <c r="I70" s="92" t="n"/>
+      <c r="J70" s="93" t="n"/>
+      <c r="K70" s="61" t="n"/>
+      <c r="L70" s="62" t="n"/>
+      <c r="M70" s="59">
         <f>IF(I70="","",ROUND(I70-E70,2))</f>
         <v/>
       </c>
-      <c r="L70" s="60">
+      <c r="N70" s="60">
         <f>IF(J70="","",J70-F70)</f>
         <v/>
       </c>
-      <c r="M70" s="56" t="n"/>
-      <c r="N70" s="56" t="n"/>
+      <c r="O70" s="56" t="n"/>
+      <c r="P70" s="56" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="47">
       <c r="A71" s="54" t="n"/>
@@ -2795,18 +2974,20 @@
       <c r="E71" s="59" t="n"/>
       <c r="F71" s="60" t="n"/>
       <c r="G71" s="54" t="n"/>
-      <c r="I71" s="61" t="n"/>
-      <c r="J71" s="62" t="n"/>
-      <c r="K71" s="59">
+      <c r="I71" s="92" t="n"/>
+      <c r="J71" s="93" t="n"/>
+      <c r="K71" s="61" t="n"/>
+      <c r="L71" s="62" t="n"/>
+      <c r="M71" s="59">
         <f>IF(I71="","",ROUND(I71-E71,2))</f>
         <v/>
       </c>
-      <c r="L71" s="60">
+      <c r="N71" s="60">
         <f>IF(J71="","",J71-F71)</f>
         <v/>
       </c>
-      <c r="M71" s="56" t="n"/>
-      <c r="N71" s="56" t="n"/>
+      <c r="O71" s="56" t="n"/>
+      <c r="P71" s="56" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="47">
       <c r="A72" s="54" t="n"/>
@@ -2816,18 +2997,20 @@
       <c r="E72" s="59" t="n"/>
       <c r="F72" s="60" t="n"/>
       <c r="G72" s="54" t="n"/>
-      <c r="I72" s="61" t="n"/>
-      <c r="J72" s="62" t="n"/>
-      <c r="K72" s="59">
+      <c r="I72" s="92" t="n"/>
+      <c r="J72" s="93" t="n"/>
+      <c r="K72" s="61" t="n"/>
+      <c r="L72" s="62" t="n"/>
+      <c r="M72" s="59">
         <f>IF(I72="","",ROUND(I72-E72,2))</f>
         <v/>
       </c>
-      <c r="L72" s="60">
+      <c r="N72" s="60">
         <f>IF(J72="","",J72-F72)</f>
         <v/>
       </c>
-      <c r="M72" s="56" t="n"/>
-      <c r="N72" s="56" t="n"/>
+      <c r="O72" s="56" t="n"/>
+      <c r="P72" s="56" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="47">
       <c r="A73" s="54" t="n"/>
@@ -2837,18 +3020,20 @@
       <c r="E73" s="59" t="n"/>
       <c r="F73" s="60" t="n"/>
       <c r="G73" s="54" t="n"/>
-      <c r="I73" s="61" t="n"/>
-      <c r="J73" s="62" t="n"/>
-      <c r="K73" s="59">
+      <c r="I73" s="92" t="n"/>
+      <c r="J73" s="93" t="n"/>
+      <c r="K73" s="61" t="n"/>
+      <c r="L73" s="62" t="n"/>
+      <c r="M73" s="59">
         <f>IF(I73="","",ROUND(I73-E73,2))</f>
         <v/>
       </c>
-      <c r="L73" s="60">
+      <c r="N73" s="60">
         <f>IF(J73="","",J73-F73)</f>
         <v/>
       </c>
-      <c r="M73" s="56" t="n"/>
-      <c r="N73" s="56" t="n"/>
+      <c r="O73" s="56" t="n"/>
+      <c r="P73" s="56" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" s="47">
       <c r="A74" s="54" t="n"/>
@@ -2858,18 +3043,20 @@
       <c r="E74" s="59" t="n"/>
       <c r="F74" s="60" t="n"/>
       <c r="G74" s="54" t="n"/>
-      <c r="I74" s="61" t="n"/>
-      <c r="J74" s="62" t="n"/>
-      <c r="K74" s="59">
+      <c r="I74" s="92" t="n"/>
+      <c r="J74" s="93" t="n"/>
+      <c r="K74" s="61" t="n"/>
+      <c r="L74" s="62" t="n"/>
+      <c r="M74" s="59">
         <f>IF(I74="","",ROUND(I74-E74,2))</f>
         <v/>
       </c>
-      <c r="L74" s="60">
+      <c r="N74" s="60">
         <f>IF(J74="","",J74-F74)</f>
         <v/>
       </c>
-      <c r="M74" s="56" t="n"/>
-      <c r="N74" s="56" t="n"/>
+      <c r="O74" s="56" t="n"/>
+      <c r="P74" s="56" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="47">
       <c r="A75" s="54" t="n"/>
@@ -2879,18 +3066,20 @@
       <c r="E75" s="59" t="n"/>
       <c r="F75" s="60" t="n"/>
       <c r="G75" s="54" t="n"/>
-      <c r="I75" s="61" t="n"/>
-      <c r="J75" s="62" t="n"/>
-      <c r="K75" s="59">
+      <c r="I75" s="92" t="n"/>
+      <c r="J75" s="93" t="n"/>
+      <c r="K75" s="61" t="n"/>
+      <c r="L75" s="62" t="n"/>
+      <c r="M75" s="59">
         <f>IF(I75="","",ROUND(I75-E75,2))</f>
         <v/>
       </c>
-      <c r="L75" s="60">
+      <c r="N75" s="60">
         <f>IF(J75="","",J75-F75)</f>
         <v/>
       </c>
-      <c r="M75" s="56" t="n"/>
-      <c r="N75" s="56" t="n"/>
+      <c r="O75" s="56" t="n"/>
+      <c r="P75" s="56" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="47">
       <c r="A76" s="54" t="n"/>
@@ -2900,18 +3089,20 @@
       <c r="E76" s="59" t="n"/>
       <c r="F76" s="60" t="n"/>
       <c r="G76" s="54" t="n"/>
-      <c r="I76" s="61" t="n"/>
-      <c r="J76" s="62" t="n"/>
-      <c r="K76" s="59">
+      <c r="I76" s="92" t="n"/>
+      <c r="J76" s="93" t="n"/>
+      <c r="K76" s="61" t="n"/>
+      <c r="L76" s="62" t="n"/>
+      <c r="M76" s="59">
         <f>IF(I76="","",ROUND(I76-E76,2))</f>
         <v/>
       </c>
-      <c r="L76" s="60">
+      <c r="N76" s="60">
         <f>IF(J76="","",J76-F76)</f>
         <v/>
       </c>
-      <c r="M76" s="56" t="n"/>
-      <c r="N76" s="56" t="n"/>
+      <c r="O76" s="56" t="n"/>
+      <c r="P76" s="56" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="47">
       <c r="A77" s="54" t="n"/>
@@ -2921,18 +3112,20 @@
       <c r="E77" s="59" t="n"/>
       <c r="F77" s="60" t="n"/>
       <c r="G77" s="54" t="n"/>
-      <c r="I77" s="61" t="n"/>
-      <c r="J77" s="62" t="n"/>
-      <c r="K77" s="59">
+      <c r="I77" s="92" t="n"/>
+      <c r="J77" s="93" t="n"/>
+      <c r="K77" s="61" t="n"/>
+      <c r="L77" s="62" t="n"/>
+      <c r="M77" s="59">
         <f>IF(I77="","",ROUND(I77-E77,2))</f>
         <v/>
       </c>
-      <c r="L77" s="60">
+      <c r="N77" s="60">
         <f>IF(J77="","",J77-F77)</f>
         <v/>
       </c>
-      <c r="M77" s="56" t="n"/>
-      <c r="N77" s="56" t="n"/>
+      <c r="O77" s="56" t="n"/>
+      <c r="P77" s="56" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="47">
       <c r="A78" s="54" t="n"/>
@@ -2942,18 +3135,20 @@
       <c r="E78" s="59" t="n"/>
       <c r="F78" s="60" t="n"/>
       <c r="G78" s="54" t="n"/>
-      <c r="I78" s="61" t="n"/>
-      <c r="J78" s="62" t="n"/>
-      <c r="K78" s="59">
+      <c r="I78" s="92" t="n"/>
+      <c r="J78" s="93" t="n"/>
+      <c r="K78" s="61" t="n"/>
+      <c r="L78" s="62" t="n"/>
+      <c r="M78" s="59">
         <f>IF(I78="","",ROUND(I78-E78,2))</f>
         <v/>
       </c>
-      <c r="L78" s="60">
+      <c r="N78" s="60">
         <f>IF(J78="","",J78-F78)</f>
         <v/>
       </c>
-      <c r="M78" s="56" t="n"/>
-      <c r="N78" s="56" t="n"/>
+      <c r="O78" s="56" t="n"/>
+      <c r="P78" s="56" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="47">
       <c r="A79" s="54" t="n"/>
@@ -2963,18 +3158,20 @@
       <c r="E79" s="59" t="n"/>
       <c r="F79" s="60" t="n"/>
       <c r="G79" s="54" t="n"/>
-      <c r="I79" s="61" t="n"/>
-      <c r="J79" s="62" t="n"/>
-      <c r="K79" s="59">
+      <c r="I79" s="92" t="n"/>
+      <c r="J79" s="93" t="n"/>
+      <c r="K79" s="61" t="n"/>
+      <c r="L79" s="62" t="n"/>
+      <c r="M79" s="59">
         <f>IF(I79="","",ROUND(I79-E79,2))</f>
         <v/>
       </c>
-      <c r="L79" s="60">
+      <c r="N79" s="60">
         <f>IF(J79="","",J79-F79)</f>
         <v/>
       </c>
-      <c r="M79" s="56" t="n"/>
-      <c r="N79" s="56" t="n"/>
+      <c r="O79" s="56" t="n"/>
+      <c r="P79" s="56" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="47">
       <c r="A80" s="54" t="n"/>
@@ -2984,18 +3181,20 @@
       <c r="E80" s="59" t="n"/>
       <c r="F80" s="60" t="n"/>
       <c r="G80" s="54" t="n"/>
-      <c r="I80" s="61" t="n"/>
-      <c r="J80" s="62" t="n"/>
-      <c r="K80" s="59">
+      <c r="I80" s="92" t="n"/>
+      <c r="J80" s="93" t="n"/>
+      <c r="K80" s="61" t="n"/>
+      <c r="L80" s="62" t="n"/>
+      <c r="M80" s="59">
         <f>IF(I80="","",ROUND(I80-E80,2))</f>
         <v/>
       </c>
-      <c r="L80" s="60">
+      <c r="N80" s="60">
         <f>IF(J80="","",J80-F80)</f>
         <v/>
       </c>
-      <c r="M80" s="56" t="n"/>
-      <c r="N80" s="56" t="n"/>
+      <c r="O80" s="56" t="n"/>
+      <c r="P80" s="56" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="47">
       <c r="A81" s="54" t="n"/>
@@ -3005,18 +3204,20 @@
       <c r="E81" s="59" t="n"/>
       <c r="F81" s="60" t="n"/>
       <c r="G81" s="54" t="n"/>
-      <c r="I81" s="61" t="n"/>
-      <c r="J81" s="62" t="n"/>
-      <c r="K81" s="59">
+      <c r="I81" s="92" t="n"/>
+      <c r="J81" s="93" t="n"/>
+      <c r="K81" s="61" t="n"/>
+      <c r="L81" s="62" t="n"/>
+      <c r="M81" s="59">
         <f>IF(I81="","",ROUND(I81-E81,2))</f>
         <v/>
       </c>
-      <c r="L81" s="60">
+      <c r="N81" s="60">
         <f>IF(J81="","",J81-F81)</f>
         <v/>
       </c>
-      <c r="M81" s="56" t="n"/>
-      <c r="N81" s="56" t="n"/>
+      <c r="O81" s="56" t="n"/>
+      <c r="P81" s="56" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1" s="47">
       <c r="A82" s="54" t="n"/>
@@ -3026,18 +3227,20 @@
       <c r="E82" s="59" t="n"/>
       <c r="F82" s="60" t="n"/>
       <c r="G82" s="54" t="n"/>
-      <c r="I82" s="61" t="n"/>
-      <c r="J82" s="62" t="n"/>
-      <c r="K82" s="59">
+      <c r="I82" s="92" t="n"/>
+      <c r="J82" s="93" t="n"/>
+      <c r="K82" s="61" t="n"/>
+      <c r="L82" s="62" t="n"/>
+      <c r="M82" s="59">
         <f>IF(I82="","",ROUND(I82-E82,2))</f>
         <v/>
       </c>
-      <c r="L82" s="60">
+      <c r="N82" s="60">
         <f>IF(J82="","",J82-F82)</f>
         <v/>
       </c>
-      <c r="M82" s="56" t="n"/>
-      <c r="N82" s="56" t="n"/>
+      <c r="O82" s="56" t="n"/>
+      <c r="P82" s="56" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1" s="47">
       <c r="A83" s="54" t="n"/>
@@ -3047,18 +3250,20 @@
       <c r="E83" s="59" t="n"/>
       <c r="F83" s="60" t="n"/>
       <c r="G83" s="54" t="n"/>
-      <c r="I83" s="61" t="n"/>
-      <c r="J83" s="62" t="n"/>
-      <c r="K83" s="59">
+      <c r="I83" s="92" t="n"/>
+      <c r="J83" s="93" t="n"/>
+      <c r="K83" s="61" t="n"/>
+      <c r="L83" s="62" t="n"/>
+      <c r="M83" s="59">
         <f>IF(I83="","",ROUND(I83-E83,2))</f>
         <v/>
       </c>
-      <c r="L83" s="60">
+      <c r="N83" s="60">
         <f>IF(J83="","",J83-F83)</f>
         <v/>
       </c>
-      <c r="M83" s="56" t="n"/>
-      <c r="N83" s="56" t="n"/>
+      <c r="O83" s="56" t="n"/>
+      <c r="P83" s="56" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="47">
       <c r="A84" s="54" t="n"/>
@@ -3068,18 +3273,20 @@
       <c r="E84" s="59" t="n"/>
       <c r="F84" s="60" t="n"/>
       <c r="G84" s="54" t="n"/>
-      <c r="I84" s="61" t="n"/>
-      <c r="J84" s="62" t="n"/>
-      <c r="K84" s="59">
+      <c r="I84" s="92" t="n"/>
+      <c r="J84" s="93" t="n"/>
+      <c r="K84" s="61" t="n"/>
+      <c r="L84" s="62" t="n"/>
+      <c r="M84" s="59">
         <f>IF(I84="","",ROUND(I84-E84,2))</f>
         <v/>
       </c>
-      <c r="L84" s="60">
+      <c r="N84" s="60">
         <f>IF(J84="","",J84-F84)</f>
         <v/>
       </c>
-      <c r="M84" s="56" t="n"/>
-      <c r="N84" s="56" t="n"/>
+      <c r="O84" s="56" t="n"/>
+      <c r="P84" s="56" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="47">
       <c r="A85" s="54" t="n"/>
@@ -3089,18 +3296,20 @@
       <c r="E85" s="59" t="n"/>
       <c r="F85" s="60" t="n"/>
       <c r="G85" s="54" t="n"/>
-      <c r="I85" s="61" t="n"/>
-      <c r="J85" s="62" t="n"/>
-      <c r="K85" s="59">
+      <c r="I85" s="92" t="n"/>
+      <c r="J85" s="93" t="n"/>
+      <c r="K85" s="61" t="n"/>
+      <c r="L85" s="62" t="n"/>
+      <c r="M85" s="59">
         <f>IF(I85="","",ROUND(I85-E85,2))</f>
         <v/>
       </c>
-      <c r="L85" s="60">
+      <c r="N85" s="60">
         <f>IF(J85="","",J85-F85)</f>
         <v/>
       </c>
-      <c r="M85" s="56" t="n"/>
-      <c r="N85" s="56" t="n"/>
+      <c r="O85" s="56" t="n"/>
+      <c r="P85" s="56" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="47">
       <c r="A86" s="54" t="n"/>
@@ -3110,18 +3319,20 @@
       <c r="E86" s="59" t="n"/>
       <c r="F86" s="60" t="n"/>
       <c r="G86" s="54" t="n"/>
-      <c r="I86" s="61" t="n"/>
-      <c r="J86" s="62" t="n"/>
-      <c r="K86" s="59">
+      <c r="I86" s="92" t="n"/>
+      <c r="J86" s="93" t="n"/>
+      <c r="K86" s="61" t="n"/>
+      <c r="L86" s="62" t="n"/>
+      <c r="M86" s="59">
         <f>IF(I86="","",ROUND(I86-E86,2))</f>
         <v/>
       </c>
-      <c r="L86" s="60">
+      <c r="N86" s="60">
         <f>IF(J86="","",J86-F86)</f>
         <v/>
       </c>
-      <c r="M86" s="56" t="n"/>
-      <c r="N86" s="56" t="n"/>
+      <c r="O86" s="56" t="n"/>
+      <c r="P86" s="56" t="n"/>
     </row>
     <row r="87" ht="15" customHeight="1" s="47">
       <c r="A87" s="54" t="n"/>
@@ -3131,18 +3342,20 @@
       <c r="E87" s="59" t="n"/>
       <c r="F87" s="60" t="n"/>
       <c r="G87" s="54" t="n"/>
-      <c r="I87" s="61" t="n"/>
-      <c r="J87" s="62" t="n"/>
-      <c r="K87" s="59">
+      <c r="I87" s="92" t="n"/>
+      <c r="J87" s="93" t="n"/>
+      <c r="K87" s="61" t="n"/>
+      <c r="L87" s="62" t="n"/>
+      <c r="M87" s="59">
         <f>IF(I87="","",ROUND(I87-E87,2))</f>
         <v/>
       </c>
-      <c r="L87" s="60">
+      <c r="N87" s="60">
         <f>IF(J87="","",J87-F87)</f>
         <v/>
       </c>
-      <c r="M87" s="56" t="n"/>
-      <c r="N87" s="56" t="n"/>
+      <c r="O87" s="56" t="n"/>
+      <c r="P87" s="56" t="n"/>
     </row>
     <row r="88" ht="15" customHeight="1" s="47">
       <c r="A88" s="54" t="n"/>
@@ -3152,18 +3365,20 @@
       <c r="E88" s="59" t="n"/>
       <c r="F88" s="60" t="n"/>
       <c r="G88" s="54" t="n"/>
-      <c r="I88" s="61" t="n"/>
-      <c r="J88" s="62" t="n"/>
-      <c r="K88" s="59">
+      <c r="I88" s="92" t="n"/>
+      <c r="J88" s="93" t="n"/>
+      <c r="K88" s="61" t="n"/>
+      <c r="L88" s="62" t="n"/>
+      <c r="M88" s="59">
         <f>IF(I88="","",ROUND(I88-E88,2))</f>
         <v/>
       </c>
-      <c r="L88" s="60">
+      <c r="N88" s="60">
         <f>IF(J88="","",J88-F88)</f>
         <v/>
       </c>
-      <c r="M88" s="56" t="n"/>
-      <c r="N88" s="56" t="n"/>
+      <c r="O88" s="56" t="n"/>
+      <c r="P88" s="56" t="n"/>
     </row>
     <row r="89" ht="15" customHeight="1" s="47">
       <c r="A89" s="54" t="n"/>
@@ -3173,18 +3388,20 @@
       <c r="E89" s="59" t="n"/>
       <c r="F89" s="60" t="n"/>
       <c r="G89" s="54" t="n"/>
-      <c r="I89" s="61" t="n"/>
-      <c r="J89" s="62" t="n"/>
-      <c r="K89" s="59">
+      <c r="I89" s="92" t="n"/>
+      <c r="J89" s="93" t="n"/>
+      <c r="K89" s="61" t="n"/>
+      <c r="L89" s="62" t="n"/>
+      <c r="M89" s="59">
         <f>IF(I89="","",ROUND(I89-E89,2))</f>
         <v/>
       </c>
-      <c r="L89" s="60">
+      <c r="N89" s="60">
         <f>IF(J89="","",J89-F89)</f>
         <v/>
       </c>
-      <c r="M89" s="56" t="n"/>
-      <c r="N89" s="56" t="n"/>
+      <c r="O89" s="56" t="n"/>
+      <c r="P89" s="56" t="n"/>
     </row>
     <row r="90" ht="15" customHeight="1" s="47">
       <c r="A90" s="54" t="n"/>
@@ -3194,18 +3411,20 @@
       <c r="E90" s="59" t="n"/>
       <c r="F90" s="60" t="n"/>
       <c r="G90" s="54" t="n"/>
-      <c r="I90" s="61" t="n"/>
-      <c r="J90" s="62" t="n"/>
-      <c r="K90" s="59">
+      <c r="I90" s="92" t="n"/>
+      <c r="J90" s="93" t="n"/>
+      <c r="K90" s="61" t="n"/>
+      <c r="L90" s="62" t="n"/>
+      <c r="M90" s="59">
         <f>IF(I90="","",ROUND(I90-E90,2))</f>
         <v/>
       </c>
-      <c r="L90" s="60">
+      <c r="N90" s="60">
         <f>IF(J90="","",J90-F90)</f>
         <v/>
       </c>
-      <c r="M90" s="56" t="n"/>
-      <c r="N90" s="56" t="n"/>
+      <c r="O90" s="56" t="n"/>
+      <c r="P90" s="56" t="n"/>
     </row>
     <row r="91" ht="15" customHeight="1" s="47">
       <c r="A91" s="54" t="n"/>
@@ -3215,18 +3434,20 @@
       <c r="E91" s="59" t="n"/>
       <c r="F91" s="60" t="n"/>
       <c r="G91" s="54" t="n"/>
-      <c r="I91" s="61" t="n"/>
-      <c r="J91" s="62" t="n"/>
-      <c r="K91" s="59">
+      <c r="I91" s="92" t="n"/>
+      <c r="J91" s="93" t="n"/>
+      <c r="K91" s="61" t="n"/>
+      <c r="L91" s="62" t="n"/>
+      <c r="M91" s="59">
         <f>IF(I91="","",ROUND(I91-E91,2))</f>
         <v/>
       </c>
-      <c r="L91" s="60">
+      <c r="N91" s="60">
         <f>IF(J91="","",J91-F91)</f>
         <v/>
       </c>
-      <c r="M91" s="56" t="n"/>
-      <c r="N91" s="56" t="n"/>
+      <c r="O91" s="56" t="n"/>
+      <c r="P91" s="56" t="n"/>
     </row>
     <row r="92" ht="15" customHeight="1" s="47">
       <c r="A92" s="54" t="n"/>
@@ -3236,18 +3457,20 @@
       <c r="E92" s="59" t="n"/>
       <c r="F92" s="60" t="n"/>
       <c r="G92" s="54" t="n"/>
-      <c r="I92" s="61" t="n"/>
-      <c r="J92" s="62" t="n"/>
-      <c r="K92" s="59">
+      <c r="I92" s="92" t="n"/>
+      <c r="J92" s="93" t="n"/>
+      <c r="K92" s="61" t="n"/>
+      <c r="L92" s="62" t="n"/>
+      <c r="M92" s="59">
         <f>IF(I92="","",ROUND(I92-E92,2))</f>
         <v/>
       </c>
-      <c r="L92" s="60">
+      <c r="N92" s="60">
         <f>IF(J92="","",J92-F92)</f>
         <v/>
       </c>
-      <c r="M92" s="56" t="n"/>
-      <c r="N92" s="56" t="n"/>
+      <c r="O92" s="56" t="n"/>
+      <c r="P92" s="56" t="n"/>
     </row>
     <row r="93" ht="15" customHeight="1" s="47">
       <c r="A93" s="54" t="n"/>
@@ -3257,18 +3480,20 @@
       <c r="E93" s="59" t="n"/>
       <c r="F93" s="60" t="n"/>
       <c r="G93" s="54" t="n"/>
-      <c r="I93" s="61" t="n"/>
-      <c r="J93" s="62" t="n"/>
-      <c r="K93" s="59">
+      <c r="I93" s="92" t="n"/>
+      <c r="J93" s="93" t="n"/>
+      <c r="K93" s="61" t="n"/>
+      <c r="L93" s="62" t="n"/>
+      <c r="M93" s="59">
         <f>IF(I93="","",ROUND(I93-E93,2))</f>
         <v/>
       </c>
-      <c r="L93" s="60">
+      <c r="N93" s="60">
         <f>IF(J93="","",J93-F93)</f>
         <v/>
       </c>
-      <c r="M93" s="56" t="n"/>
-      <c r="N93" s="56" t="n"/>
+      <c r="O93" s="56" t="n"/>
+      <c r="P93" s="56" t="n"/>
     </row>
     <row r="94" ht="15" customHeight="1" s="47">
       <c r="A94" s="54" t="n"/>
@@ -3278,18 +3503,20 @@
       <c r="E94" s="59" t="n"/>
       <c r="F94" s="60" t="n"/>
       <c r="G94" s="54" t="n"/>
-      <c r="I94" s="61" t="n"/>
-      <c r="J94" s="62" t="n"/>
-      <c r="K94" s="59">
+      <c r="I94" s="92" t="n"/>
+      <c r="J94" s="93" t="n"/>
+      <c r="K94" s="61" t="n"/>
+      <c r="L94" s="62" t="n"/>
+      <c r="M94" s="59">
         <f>IF(I94="","",ROUND(I94-E94,2))</f>
         <v/>
       </c>
-      <c r="L94" s="60">
+      <c r="N94" s="60">
         <f>IF(J94="","",J94-F94)</f>
         <v/>
       </c>
-      <c r="M94" s="56" t="n"/>
-      <c r="N94" s="56" t="n"/>
+      <c r="O94" s="56" t="n"/>
+      <c r="P94" s="56" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="47">
       <c r="A95" s="54" t="n"/>
@@ -3299,18 +3526,20 @@
       <c r="E95" s="59" t="n"/>
       <c r="F95" s="60" t="n"/>
       <c r="G95" s="54" t="n"/>
-      <c r="I95" s="61" t="n"/>
-      <c r="J95" s="62" t="n"/>
-      <c r="K95" s="59">
+      <c r="I95" s="92" t="n"/>
+      <c r="J95" s="93" t="n"/>
+      <c r="K95" s="61" t="n"/>
+      <c r="L95" s="62" t="n"/>
+      <c r="M95" s="59">
         <f>IF(I95="","",ROUND(I95-E95,2))</f>
         <v/>
       </c>
-      <c r="L95" s="60">
+      <c r="N95" s="60">
         <f>IF(J95="","",J95-F95)</f>
         <v/>
       </c>
-      <c r="M95" s="56" t="n"/>
-      <c r="N95" s="56" t="n"/>
+      <c r="O95" s="56" t="n"/>
+      <c r="P95" s="56" t="n"/>
     </row>
     <row r="96" ht="15" customHeight="1" s="47">
       <c r="A96" s="54" t="n"/>
@@ -3320,18 +3549,20 @@
       <c r="E96" s="59" t="n"/>
       <c r="F96" s="60" t="n"/>
       <c r="G96" s="54" t="n"/>
-      <c r="I96" s="61" t="n"/>
-      <c r="J96" s="62" t="n"/>
-      <c r="K96" s="59">
+      <c r="I96" s="92" t="n"/>
+      <c r="J96" s="93" t="n"/>
+      <c r="K96" s="61" t="n"/>
+      <c r="L96" s="62" t="n"/>
+      <c r="M96" s="59">
         <f>IF(I96="","",ROUND(I96-E96,2))</f>
         <v/>
       </c>
-      <c r="L96" s="60">
+      <c r="N96" s="60">
         <f>IF(J96="","",J96-F96)</f>
         <v/>
       </c>
-      <c r="M96" s="56" t="n"/>
-      <c r="N96" s="56" t="n"/>
+      <c r="O96" s="56" t="n"/>
+      <c r="P96" s="56" t="n"/>
     </row>
     <row r="97" ht="15" customHeight="1" s="47">
       <c r="A97" s="54" t="n"/>
@@ -3341,18 +3572,20 @@
       <c r="E97" s="59" t="n"/>
       <c r="F97" s="60" t="n"/>
       <c r="G97" s="54" t="n"/>
-      <c r="I97" s="61" t="n"/>
-      <c r="J97" s="62" t="n"/>
-      <c r="K97" s="59">
+      <c r="I97" s="92" t="n"/>
+      <c r="J97" s="93" t="n"/>
+      <c r="K97" s="61" t="n"/>
+      <c r="L97" s="62" t="n"/>
+      <c r="M97" s="59">
         <f>IF(I97="","",ROUND(I97-E97,2))</f>
         <v/>
       </c>
-      <c r="L97" s="60">
+      <c r="N97" s="60">
         <f>IF(J97="","",J97-F97)</f>
         <v/>
       </c>
-      <c r="M97" s="56" t="n"/>
-      <c r="N97" s="56" t="n"/>
+      <c r="O97" s="56" t="n"/>
+      <c r="P97" s="56" t="n"/>
     </row>
     <row r="98" ht="15" customHeight="1" s="47">
       <c r="A98" s="54" t="n"/>
@@ -3362,18 +3595,20 @@
       <c r="E98" s="59" t="n"/>
       <c r="F98" s="60" t="n"/>
       <c r="G98" s="54" t="n"/>
-      <c r="I98" s="61" t="n"/>
-      <c r="J98" s="62" t="n"/>
-      <c r="K98" s="59">
+      <c r="I98" s="92" t="n"/>
+      <c r="J98" s="93" t="n"/>
+      <c r="K98" s="61" t="n"/>
+      <c r="L98" s="62" t="n"/>
+      <c r="M98" s="59">
         <f>IF(I98="","",ROUND(I98-E98,2))</f>
         <v/>
       </c>
-      <c r="L98" s="60">
+      <c r="N98" s="60">
         <f>IF(J98="","",J98-F98)</f>
         <v/>
       </c>
-      <c r="M98" s="56" t="n"/>
-      <c r="N98" s="56" t="n"/>
+      <c r="O98" s="56" t="n"/>
+      <c r="P98" s="56" t="n"/>
     </row>
     <row r="99" ht="15" customHeight="1" s="47">
       <c r="A99" s="54" t="n"/>
@@ -3383,18 +3618,20 @@
       <c r="E99" s="59" t="n"/>
       <c r="F99" s="60" t="n"/>
       <c r="G99" s="54" t="n"/>
-      <c r="I99" s="61" t="n"/>
-      <c r="J99" s="62" t="n"/>
-      <c r="K99" s="59">
+      <c r="I99" s="92" t="n"/>
+      <c r="J99" s="93" t="n"/>
+      <c r="K99" s="61" t="n"/>
+      <c r="L99" s="62" t="n"/>
+      <c r="M99" s="59">
         <f>IF(I99="","",ROUND(I99-E99,2))</f>
         <v/>
       </c>
-      <c r="L99" s="60">
+      <c r="N99" s="60">
         <f>IF(J99="","",J99-F99)</f>
         <v/>
       </c>
-      <c r="M99" s="56" t="n"/>
-      <c r="N99" s="56" t="n"/>
+      <c r="O99" s="56" t="n"/>
+      <c r="P99" s="56" t="n"/>
     </row>
     <row r="100" ht="15" customHeight="1" s="47">
       <c r="A100" s="54" t="n"/>
@@ -3404,18 +3641,20 @@
       <c r="E100" s="59" t="n"/>
       <c r="F100" s="60" t="n"/>
       <c r="G100" s="54" t="n"/>
-      <c r="I100" s="61" t="n"/>
-      <c r="J100" s="62" t="n"/>
-      <c r="K100" s="59">
+      <c r="I100" s="92" t="n"/>
+      <c r="J100" s="93" t="n"/>
+      <c r="K100" s="61" t="n"/>
+      <c r="L100" s="62" t="n"/>
+      <c r="M100" s="59">
         <f>IF(I100="","",ROUND(I100-E100,2))</f>
         <v/>
       </c>
-      <c r="L100" s="60">
+      <c r="N100" s="60">
         <f>IF(J100="","",J100-F100)</f>
         <v/>
       </c>
-      <c r="M100" s="56" t="n"/>
-      <c r="N100" s="56" t="n"/>
+      <c r="O100" s="56" t="n"/>
+      <c r="P100" s="56" t="n"/>
     </row>
     <row r="101" ht="15" customHeight="1" s="47">
       <c r="A101" s="54" t="n"/>
@@ -3425,18 +3664,20 @@
       <c r="E101" s="59" t="n"/>
       <c r="F101" s="60" t="n"/>
       <c r="G101" s="54" t="n"/>
-      <c r="I101" s="61" t="n"/>
-      <c r="J101" s="62" t="n"/>
-      <c r="K101" s="59">
+      <c r="I101" s="92" t="n"/>
+      <c r="J101" s="93" t="n"/>
+      <c r="K101" s="61" t="n"/>
+      <c r="L101" s="62" t="n"/>
+      <c r="M101" s="59">
         <f>IF(I101="","",ROUND(I101-E101,2))</f>
         <v/>
       </c>
-      <c r="L101" s="60">
+      <c r="N101" s="60">
         <f>IF(J101="","",J101-F101)</f>
         <v/>
       </c>
-      <c r="M101" s="56" t="n"/>
-      <c r="N101" s="56" t="n"/>
+      <c r="O101" s="56" t="n"/>
+      <c r="P101" s="56" t="n"/>
     </row>
     <row r="102" ht="15" customHeight="1" s="47">
       <c r="A102" s="54" t="n"/>
@@ -3446,18 +3687,20 @@
       <c r="E102" s="59" t="n"/>
       <c r="F102" s="60" t="n"/>
       <c r="G102" s="54" t="n"/>
-      <c r="I102" s="61" t="n"/>
-      <c r="J102" s="62" t="n"/>
-      <c r="K102" s="59">
+      <c r="I102" s="92" t="n"/>
+      <c r="J102" s="93" t="n"/>
+      <c r="K102" s="61" t="n"/>
+      <c r="L102" s="62" t="n"/>
+      <c r="M102" s="59">
         <f>IF(I102="","",ROUND(I102-E102,2))</f>
         <v/>
       </c>
-      <c r="L102" s="60">
+      <c r="N102" s="60">
         <f>IF(J102="","",J102-F102)</f>
         <v/>
       </c>
-      <c r="M102" s="56" t="n"/>
-      <c r="N102" s="56" t="n"/>
+      <c r="O102" s="56" t="n"/>
+      <c r="P102" s="56" t="n"/>
     </row>
     <row r="103" ht="15" customHeight="1" s="47">
       <c r="A103" s="54" t="n"/>
@@ -3467,18 +3710,20 @@
       <c r="E103" s="59" t="n"/>
       <c r="F103" s="60" t="n"/>
       <c r="G103" s="54" t="n"/>
-      <c r="I103" s="61" t="n"/>
-      <c r="J103" s="62" t="n"/>
-      <c r="K103" s="59">
+      <c r="I103" s="92" t="n"/>
+      <c r="J103" s="93" t="n"/>
+      <c r="K103" s="61" t="n"/>
+      <c r="L103" s="62" t="n"/>
+      <c r="M103" s="59">
         <f>IF(I103="","",ROUND(I103-E103,2))</f>
         <v/>
       </c>
-      <c r="L103" s="60">
+      <c r="N103" s="60">
         <f>IF(J103="","",J103-F103)</f>
         <v/>
       </c>
-      <c r="M103" s="56" t="n"/>
-      <c r="N103" s="56" t="n"/>
+      <c r="O103" s="56" t="n"/>
+      <c r="P103" s="56" t="n"/>
     </row>
     <row r="104" ht="15" customHeight="1" s="47">
       <c r="A104" s="54" t="n"/>
@@ -3488,18 +3733,20 @@
       <c r="E104" s="59" t="n"/>
       <c r="F104" s="60" t="n"/>
       <c r="G104" s="54" t="n"/>
-      <c r="I104" s="61" t="n"/>
-      <c r="J104" s="62" t="n"/>
-      <c r="K104" s="59">
+      <c r="I104" s="92" t="n"/>
+      <c r="J104" s="93" t="n"/>
+      <c r="K104" s="61" t="n"/>
+      <c r="L104" s="62" t="n"/>
+      <c r="M104" s="59">
         <f>IF(I104="","",ROUND(I104-E104,2))</f>
         <v/>
       </c>
-      <c r="L104" s="60">
+      <c r="N104" s="60">
         <f>IF(J104="","",J104-F104)</f>
         <v/>
       </c>
-      <c r="M104" s="56" t="n"/>
-      <c r="N104" s="56" t="n"/>
+      <c r="O104" s="56" t="n"/>
+      <c r="P104" s="56" t="n"/>
     </row>
     <row r="105" ht="15" customHeight="1" s="47">
       <c r="A105" s="54" t="n"/>
@@ -3509,18 +3756,20 @@
       <c r="E105" s="59" t="n"/>
       <c r="F105" s="60" t="n"/>
       <c r="G105" s="54" t="n"/>
-      <c r="I105" s="61" t="n"/>
-      <c r="J105" s="62" t="n"/>
-      <c r="K105" s="59">
+      <c r="I105" s="92" t="n"/>
+      <c r="J105" s="93" t="n"/>
+      <c r="K105" s="61" t="n"/>
+      <c r="L105" s="62" t="n"/>
+      <c r="M105" s="59">
         <f>IF(I105="","",ROUND(I105-E105,2))</f>
         <v/>
       </c>
-      <c r="L105" s="60">
+      <c r="N105" s="60">
         <f>IF(J105="","",J105-F105)</f>
         <v/>
       </c>
-      <c r="M105" s="56" t="n"/>
-      <c r="N105" s="56" t="n"/>
+      <c r="O105" s="56" t="n"/>
+      <c r="P105" s="56" t="n"/>
     </row>
     <row r="106" ht="15" customHeight="1" s="47">
       <c r="A106" s="54" t="n"/>
@@ -3530,18 +3779,20 @@
       <c r="E106" s="59" t="n"/>
       <c r="F106" s="60" t="n"/>
       <c r="G106" s="54" t="n"/>
-      <c r="I106" s="61" t="n"/>
-      <c r="J106" s="62" t="n"/>
-      <c r="K106" s="59">
+      <c r="I106" s="92" t="n"/>
+      <c r="J106" s="93" t="n"/>
+      <c r="K106" s="61" t="n"/>
+      <c r="L106" s="62" t="n"/>
+      <c r="M106" s="59">
         <f>IF(I106="","",ROUND(I106-E106,2))</f>
         <v/>
       </c>
-      <c r="L106" s="60">
+      <c r="N106" s="60">
         <f>IF(J106="","",J106-F106)</f>
         <v/>
       </c>
-      <c r="M106" s="56" t="n"/>
-      <c r="N106" s="56" t="n"/>
+      <c r="O106" s="56" t="n"/>
+      <c r="P106" s="56" t="n"/>
     </row>
     <row r="107" ht="15" customHeight="1" s="47">
       <c r="A107" s="54" t="n"/>
@@ -3551,18 +3802,20 @@
       <c r="E107" s="59" t="n"/>
       <c r="F107" s="60" t="n"/>
       <c r="G107" s="54" t="n"/>
-      <c r="I107" s="61" t="n"/>
-      <c r="J107" s="62" t="n"/>
-      <c r="K107" s="59">
+      <c r="I107" s="92" t="n"/>
+      <c r="J107" s="93" t="n"/>
+      <c r="K107" s="61" t="n"/>
+      <c r="L107" s="62" t="n"/>
+      <c r="M107" s="59">
         <f>IF(I107="","",ROUND(I107-E107,2))</f>
         <v/>
       </c>
-      <c r="L107" s="60">
+      <c r="N107" s="60">
         <f>IF(J107="","",J107-F107)</f>
         <v/>
       </c>
-      <c r="M107" s="56" t="n"/>
-      <c r="N107" s="56" t="n"/>
+      <c r="O107" s="56" t="n"/>
+      <c r="P107" s="56" t="n"/>
     </row>
     <row r="108" ht="15" customHeight="1" s="47">
       <c r="A108" s="54" t="n"/>
@@ -3572,18 +3825,20 @@
       <c r="E108" s="59" t="n"/>
       <c r="F108" s="60" t="n"/>
       <c r="G108" s="54" t="n"/>
-      <c r="I108" s="61" t="n"/>
-      <c r="J108" s="62" t="n"/>
-      <c r="K108" s="59">
+      <c r="I108" s="92" t="n"/>
+      <c r="J108" s="93" t="n"/>
+      <c r="K108" s="61" t="n"/>
+      <c r="L108" s="62" t="n"/>
+      <c r="M108" s="59">
         <f>IF(I108="","",ROUND(I108-E108,2))</f>
         <v/>
       </c>
-      <c r="L108" s="60">
+      <c r="N108" s="60">
         <f>IF(J108="","",J108-F108)</f>
         <v/>
       </c>
-      <c r="M108" s="56" t="n"/>
-      <c r="N108" s="56" t="n"/>
+      <c r="O108" s="56" t="n"/>
+      <c r="P108" s="56" t="n"/>
     </row>
     <row r="109" ht="15" customHeight="1" s="47">
       <c r="A109" s="54" t="n"/>
@@ -3593,18 +3848,20 @@
       <c r="E109" s="59" t="n"/>
       <c r="F109" s="60" t="n"/>
       <c r="G109" s="54" t="n"/>
-      <c r="I109" s="61" t="n"/>
-      <c r="J109" s="62" t="n"/>
-      <c r="K109" s="59">
+      <c r="I109" s="92" t="n"/>
+      <c r="J109" s="93" t="n"/>
+      <c r="K109" s="61" t="n"/>
+      <c r="L109" s="62" t="n"/>
+      <c r="M109" s="59">
         <f>IF(I109="","",ROUND(I109-E109,2))</f>
         <v/>
       </c>
-      <c r="L109" s="60">
+      <c r="N109" s="60">
         <f>IF(J109="","",J109-F109)</f>
         <v/>
       </c>
-      <c r="M109" s="56" t="n"/>
-      <c r="N109" s="56" t="n"/>
+      <c r="O109" s="56" t="n"/>
+      <c r="P109" s="56" t="n"/>
     </row>
     <row r="110" ht="15" customHeight="1" s="47">
       <c r="A110" s="54" t="n"/>
@@ -3614,18 +3871,20 @@
       <c r="E110" s="59" t="n"/>
       <c r="F110" s="60" t="n"/>
       <c r="G110" s="54" t="n"/>
-      <c r="I110" s="61" t="n"/>
-      <c r="J110" s="62" t="n"/>
-      <c r="K110" s="59">
+      <c r="I110" s="92" t="n"/>
+      <c r="J110" s="93" t="n"/>
+      <c r="K110" s="61" t="n"/>
+      <c r="L110" s="62" t="n"/>
+      <c r="M110" s="59">
         <f>IF(I110="","",ROUND(I110-E110,2))</f>
         <v/>
       </c>
-      <c r="L110" s="60">
+      <c r="N110" s="60">
         <f>IF(J110="","",J110-F110)</f>
         <v/>
       </c>
-      <c r="M110" s="56" t="n"/>
-      <c r="N110" s="56" t="n"/>
+      <c r="O110" s="56" t="n"/>
+      <c r="P110" s="56" t="n"/>
     </row>
     <row r="111" ht="15" customHeight="1" s="47">
       <c r="A111" s="54" t="n"/>
@@ -3635,18 +3894,20 @@
       <c r="E111" s="59" t="n"/>
       <c r="F111" s="60" t="n"/>
       <c r="G111" s="54" t="n"/>
-      <c r="I111" s="61" t="n"/>
-      <c r="J111" s="62" t="n"/>
-      <c r="K111" s="59">
+      <c r="I111" s="92" t="n"/>
+      <c r="J111" s="93" t="n"/>
+      <c r="K111" s="61" t="n"/>
+      <c r="L111" s="62" t="n"/>
+      <c r="M111" s="59">
         <f>IF(I111="","",ROUND(I111-E111,2))</f>
         <v/>
       </c>
-      <c r="L111" s="60">
+      <c r="N111" s="60">
         <f>IF(J111="","",J111-F111)</f>
         <v/>
       </c>
-      <c r="M111" s="56" t="n"/>
-      <c r="N111" s="56" t="n"/>
+      <c r="O111" s="56" t="n"/>
+      <c r="P111" s="56" t="n"/>
     </row>
     <row r="112" ht="15" customHeight="1" s="47">
       <c r="A112" s="54" t="n"/>
@@ -3656,18 +3917,20 @@
       <c r="E112" s="59" t="n"/>
       <c r="F112" s="60" t="n"/>
       <c r="G112" s="54" t="n"/>
-      <c r="I112" s="61" t="n"/>
-      <c r="J112" s="62" t="n"/>
-      <c r="K112" s="59">
+      <c r="I112" s="92" t="n"/>
+      <c r="J112" s="93" t="n"/>
+      <c r="K112" s="61" t="n"/>
+      <c r="L112" s="62" t="n"/>
+      <c r="M112" s="59">
         <f>IF(I112="","",ROUND(I112-E112,2))</f>
         <v/>
       </c>
-      <c r="L112" s="60">
+      <c r="N112" s="60">
         <f>IF(J112="","",J112-F112)</f>
         <v/>
       </c>
-      <c r="M112" s="56" t="n"/>
-      <c r="N112" s="56" t="n"/>
+      <c r="O112" s="56" t="n"/>
+      <c r="P112" s="56" t="n"/>
     </row>
     <row r="113" ht="15" customHeight="1" s="47">
       <c r="A113" s="54" t="n"/>
@@ -3677,18 +3940,20 @@
       <c r="E113" s="59" t="n"/>
       <c r="F113" s="60" t="n"/>
       <c r="G113" s="54" t="n"/>
-      <c r="I113" s="61" t="n"/>
-      <c r="J113" s="62" t="n"/>
-      <c r="K113" s="59">
+      <c r="I113" s="92" t="n"/>
+      <c r="J113" s="93" t="n"/>
+      <c r="K113" s="61" t="n"/>
+      <c r="L113" s="62" t="n"/>
+      <c r="M113" s="59">
         <f>IF(I113="","",ROUND(I113-E113,2))</f>
         <v/>
       </c>
-      <c r="L113" s="60">
+      <c r="N113" s="60">
         <f>IF(J113="","",J113-F113)</f>
         <v/>
       </c>
-      <c r="M113" s="56" t="n"/>
-      <c r="N113" s="56" t="n"/>
+      <c r="O113" s="56" t="n"/>
+      <c r="P113" s="56" t="n"/>
     </row>
     <row r="114" ht="15" customHeight="1" s="47">
       <c r="A114" s="54" t="n"/>
@@ -3698,18 +3963,20 @@
       <c r="E114" s="59" t="n"/>
       <c r="F114" s="60" t="n"/>
       <c r="G114" s="54" t="n"/>
-      <c r="I114" s="61" t="n"/>
-      <c r="J114" s="62" t="n"/>
-      <c r="K114" s="59">
+      <c r="I114" s="92" t="n"/>
+      <c r="J114" s="93" t="n"/>
+      <c r="K114" s="61" t="n"/>
+      <c r="L114" s="62" t="n"/>
+      <c r="M114" s="59">
         <f>IF(I114="","",ROUND(I114-E114,2))</f>
         <v/>
       </c>
-      <c r="L114" s="60">
+      <c r="N114" s="60">
         <f>IF(J114="","",J114-F114)</f>
         <v/>
       </c>
-      <c r="M114" s="56" t="n"/>
-      <c r="N114" s="56" t="n"/>
+      <c r="O114" s="56" t="n"/>
+      <c r="P114" s="56" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1" s="47">
       <c r="A115" s="54" t="n"/>
@@ -3719,18 +3986,20 @@
       <c r="E115" s="59" t="n"/>
       <c r="F115" s="60" t="n"/>
       <c r="G115" s="54" t="n"/>
-      <c r="I115" s="61" t="n"/>
-      <c r="J115" s="62" t="n"/>
-      <c r="K115" s="59">
+      <c r="I115" s="92" t="n"/>
+      <c r="J115" s="93" t="n"/>
+      <c r="K115" s="61" t="n"/>
+      <c r="L115" s="62" t="n"/>
+      <c r="M115" s="59">
         <f>IF(I115="","",ROUND(I115-E115,2))</f>
         <v/>
       </c>
-      <c r="L115" s="60">
+      <c r="N115" s="60">
         <f>IF(J115="","",J115-F115)</f>
         <v/>
       </c>
-      <c r="M115" s="56" t="n"/>
-      <c r="N115" s="56" t="n"/>
+      <c r="O115" s="56" t="n"/>
+      <c r="P115" s="56" t="n"/>
     </row>
     <row r="116" ht="15" customHeight="1" s="47">
       <c r="A116" s="54" t="n"/>
@@ -3740,18 +4009,20 @@
       <c r="E116" s="59" t="n"/>
       <c r="F116" s="60" t="n"/>
       <c r="G116" s="54" t="n"/>
-      <c r="I116" s="61" t="n"/>
-      <c r="J116" s="62" t="n"/>
-      <c r="K116" s="59">
+      <c r="I116" s="92" t="n"/>
+      <c r="J116" s="93" t="n"/>
+      <c r="K116" s="61" t="n"/>
+      <c r="L116" s="62" t="n"/>
+      <c r="M116" s="59">
         <f>IF(I116="","",ROUND(I116-E116,2))</f>
         <v/>
       </c>
-      <c r="L116" s="60">
+      <c r="N116" s="60">
         <f>IF(J116="","",J116-F116)</f>
         <v/>
       </c>
-      <c r="M116" s="56" t="n"/>
-      <c r="N116" s="56" t="n"/>
+      <c r="O116" s="56" t="n"/>
+      <c r="P116" s="56" t="n"/>
     </row>
     <row r="117" ht="15" customHeight="1" s="47">
       <c r="A117" s="54" t="n"/>
@@ -3761,18 +4032,20 @@
       <c r="E117" s="59" t="n"/>
       <c r="F117" s="60" t="n"/>
       <c r="G117" s="54" t="n"/>
-      <c r="I117" s="61" t="n"/>
-      <c r="J117" s="62" t="n"/>
-      <c r="K117" s="59">
+      <c r="I117" s="92" t="n"/>
+      <c r="J117" s="93" t="n"/>
+      <c r="K117" s="61" t="n"/>
+      <c r="L117" s="62" t="n"/>
+      <c r="M117" s="59">
         <f>IF(I117="","",ROUND(I117-E117,2))</f>
         <v/>
       </c>
-      <c r="L117" s="60">
+      <c r="N117" s="60">
         <f>IF(J117="","",J117-F117)</f>
         <v/>
       </c>
-      <c r="M117" s="56" t="n"/>
-      <c r="N117" s="56" t="n"/>
+      <c r="O117" s="56" t="n"/>
+      <c r="P117" s="56" t="n"/>
     </row>
     <row r="118" ht="15" customHeight="1" s="47">
       <c r="A118" s="54" t="n"/>
@@ -3782,18 +4055,20 @@
       <c r="E118" s="59" t="n"/>
       <c r="F118" s="60" t="n"/>
       <c r="G118" s="54" t="n"/>
-      <c r="I118" s="61" t="n"/>
-      <c r="J118" s="62" t="n"/>
-      <c r="K118" s="59">
+      <c r="I118" s="92" t="n"/>
+      <c r="J118" s="93" t="n"/>
+      <c r="K118" s="61" t="n"/>
+      <c r="L118" s="62" t="n"/>
+      <c r="M118" s="59">
         <f>IF(I118="","",ROUND(I118-E118,2))</f>
         <v/>
       </c>
-      <c r="L118" s="60">
+      <c r="N118" s="60">
         <f>IF(J118="","",J118-F118)</f>
         <v/>
       </c>
-      <c r="M118" s="56" t="n"/>
-      <c r="N118" s="56" t="n"/>
+      <c r="O118" s="56" t="n"/>
+      <c r="P118" s="56" t="n"/>
     </row>
     <row r="119" ht="15" customHeight="1" s="47">
       <c r="A119" s="54" t="n"/>
@@ -3803,18 +4078,20 @@
       <c r="E119" s="59" t="n"/>
       <c r="F119" s="60" t="n"/>
       <c r="G119" s="54" t="n"/>
-      <c r="I119" s="61" t="n"/>
-      <c r="J119" s="62" t="n"/>
-      <c r="K119" s="59">
+      <c r="I119" s="92" t="n"/>
+      <c r="J119" s="93" t="n"/>
+      <c r="K119" s="61" t="n"/>
+      <c r="L119" s="62" t="n"/>
+      <c r="M119" s="59">
         <f>IF(I119="","",ROUND(I119-E119,2))</f>
         <v/>
       </c>
-      <c r="L119" s="60">
+      <c r="N119" s="60">
         <f>IF(J119="","",J119-F119)</f>
         <v/>
       </c>
-      <c r="M119" s="56" t="n"/>
-      <c r="N119" s="56" t="n"/>
+      <c r="O119" s="56" t="n"/>
+      <c r="P119" s="56" t="n"/>
     </row>
     <row r="120" ht="15" customHeight="1" s="47">
       <c r="A120" s="54" t="n"/>
@@ -3824,18 +4101,20 @@
       <c r="E120" s="59" t="n"/>
       <c r="F120" s="60" t="n"/>
       <c r="G120" s="54" t="n"/>
-      <c r="I120" s="61" t="n"/>
-      <c r="J120" s="62" t="n"/>
-      <c r="K120" s="59">
+      <c r="I120" s="92" t="n"/>
+      <c r="J120" s="93" t="n"/>
+      <c r="K120" s="61" t="n"/>
+      <c r="L120" s="62" t="n"/>
+      <c r="M120" s="59">
         <f>IF(I120="","",ROUND(I120-E120,2))</f>
         <v/>
       </c>
-      <c r="L120" s="60">
+      <c r="N120" s="60">
         <f>IF(J120="","",J120-F120)</f>
         <v/>
       </c>
-      <c r="M120" s="56" t="n"/>
-      <c r="N120" s="56" t="n"/>
+      <c r="O120" s="56" t="n"/>
+      <c r="P120" s="56" t="n"/>
     </row>
     <row r="121" ht="15" customHeight="1" s="47">
       <c r="A121" s="54" t="n"/>
@@ -3845,18 +4124,20 @@
       <c r="E121" s="59" t="n"/>
       <c r="F121" s="60" t="n"/>
       <c r="G121" s="54" t="n"/>
-      <c r="I121" s="61" t="n"/>
-      <c r="J121" s="62" t="n"/>
-      <c r="K121" s="59">
+      <c r="I121" s="92" t="n"/>
+      <c r="J121" s="93" t="n"/>
+      <c r="K121" s="61" t="n"/>
+      <c r="L121" s="62" t="n"/>
+      <c r="M121" s="59">
         <f>IF(I121="","",ROUND(I121-E121,2))</f>
         <v/>
       </c>
-      <c r="L121" s="60">
+      <c r="N121" s="60">
         <f>IF(J121="","",J121-F121)</f>
         <v/>
       </c>
-      <c r="M121" s="56" t="n"/>
-      <c r="N121" s="56" t="n"/>
+      <c r="O121" s="56" t="n"/>
+      <c r="P121" s="56" t="n"/>
     </row>
     <row r="122" ht="15" customHeight="1" s="47">
       <c r="A122" s="54" t="n"/>
@@ -3866,18 +4147,20 @@
       <c r="E122" s="59" t="n"/>
       <c r="F122" s="60" t="n"/>
       <c r="G122" s="54" t="n"/>
-      <c r="I122" s="61" t="n"/>
-      <c r="J122" s="62" t="n"/>
-      <c r="K122" s="59">
+      <c r="I122" s="92" t="n"/>
+      <c r="J122" s="93" t="n"/>
+      <c r="K122" s="61" t="n"/>
+      <c r="L122" s="62" t="n"/>
+      <c r="M122" s="59">
         <f>IF(I122="","",ROUND(I122-E122,2))</f>
         <v/>
       </c>
-      <c r="L122" s="60">
+      <c r="N122" s="60">
         <f>IF(J122="","",J122-F122)</f>
         <v/>
       </c>
-      <c r="M122" s="56" t="n"/>
-      <c r="N122" s="56" t="n"/>
+      <c r="O122" s="56" t="n"/>
+      <c r="P122" s="56" t="n"/>
     </row>
     <row r="123" ht="15" customHeight="1" s="47">
       <c r="A123" s="54" t="n"/>
@@ -3887,18 +4170,20 @@
       <c r="E123" s="59" t="n"/>
       <c r="F123" s="60" t="n"/>
       <c r="G123" s="54" t="n"/>
-      <c r="I123" s="61" t="n"/>
-      <c r="J123" s="62" t="n"/>
-      <c r="K123" s="59">
+      <c r="I123" s="92" t="n"/>
+      <c r="J123" s="93" t="n"/>
+      <c r="K123" s="61" t="n"/>
+      <c r="L123" s="62" t="n"/>
+      <c r="M123" s="59">
         <f>IF(I123="","",ROUND(I123-E123,2))</f>
         <v/>
       </c>
-      <c r="L123" s="60">
+      <c r="N123" s="60">
         <f>IF(J123="","",J123-F123)</f>
         <v/>
       </c>
-      <c r="M123" s="56" t="n"/>
-      <c r="N123" s="56" t="n"/>
+      <c r="O123" s="56" t="n"/>
+      <c r="P123" s="56" t="n"/>
     </row>
     <row r="124" ht="15" customHeight="1" s="47">
       <c r="A124" s="54" t="n"/>
@@ -3908,18 +4193,20 @@
       <c r="E124" s="59" t="n"/>
       <c r="F124" s="60" t="n"/>
       <c r="G124" s="54" t="n"/>
-      <c r="I124" s="61" t="n"/>
-      <c r="J124" s="62" t="n"/>
-      <c r="K124" s="59">
+      <c r="I124" s="92" t="n"/>
+      <c r="J124" s="93" t="n"/>
+      <c r="K124" s="61" t="n"/>
+      <c r="L124" s="62" t="n"/>
+      <c r="M124" s="59">
         <f>IF(I124="","",ROUND(I124-E124,2))</f>
         <v/>
       </c>
-      <c r="L124" s="60">
+      <c r="N124" s="60">
         <f>IF(J124="","",J124-F124)</f>
         <v/>
       </c>
-      <c r="M124" s="56" t="n"/>
-      <c r="N124" s="56" t="n"/>
+      <c r="O124" s="56" t="n"/>
+      <c r="P124" s="56" t="n"/>
     </row>
     <row r="125" ht="15" customHeight="1" s="47">
       <c r="A125" s="54" t="n"/>
@@ -3929,18 +4216,20 @@
       <c r="E125" s="59" t="n"/>
       <c r="F125" s="60" t="n"/>
       <c r="G125" s="54" t="n"/>
-      <c r="I125" s="61" t="n"/>
-      <c r="J125" s="62" t="n"/>
-      <c r="K125" s="59">
+      <c r="I125" s="92" t="n"/>
+      <c r="J125" s="93" t="n"/>
+      <c r="K125" s="61" t="n"/>
+      <c r="L125" s="62" t="n"/>
+      <c r="M125" s="59">
         <f>IF(I125="","",ROUND(I125-E125,2))</f>
         <v/>
       </c>
-      <c r="L125" s="60">
+      <c r="N125" s="60">
         <f>IF(J125="","",J125-F125)</f>
         <v/>
       </c>
-      <c r="M125" s="56" t="n"/>
-      <c r="N125" s="56" t="n"/>
+      <c r="O125" s="56" t="n"/>
+      <c r="P125" s="56" t="n"/>
     </row>
     <row r="126" ht="15" customHeight="1" s="47">
       <c r="A126" s="54" t="n"/>
@@ -3950,18 +4239,20 @@
       <c r="E126" s="59" t="n"/>
       <c r="F126" s="60" t="n"/>
       <c r="G126" s="54" t="n"/>
-      <c r="I126" s="61" t="n"/>
-      <c r="J126" s="62" t="n"/>
-      <c r="K126" s="59">
+      <c r="I126" s="92" t="n"/>
+      <c r="J126" s="93" t="n"/>
+      <c r="K126" s="61" t="n"/>
+      <c r="L126" s="62" t="n"/>
+      <c r="M126" s="59">
         <f>IF(I126="","",ROUND(I126-E126,2))</f>
         <v/>
       </c>
-      <c r="L126" s="60">
+      <c r="N126" s="60">
         <f>IF(J126="","",J126-F126)</f>
         <v/>
       </c>
-      <c r="M126" s="56" t="n"/>
-      <c r="N126" s="56" t="n"/>
+      <c r="O126" s="56" t="n"/>
+      <c r="P126" s="56" t="n"/>
     </row>
     <row r="127" ht="15" customHeight="1" s="47">
       <c r="A127" s="54" t="n"/>
@@ -3971,18 +4262,20 @@
       <c r="E127" s="59" t="n"/>
       <c r="F127" s="60" t="n"/>
       <c r="G127" s="54" t="n"/>
-      <c r="I127" s="61" t="n"/>
-      <c r="J127" s="62" t="n"/>
-      <c r="K127" s="59">
+      <c r="I127" s="92" t="n"/>
+      <c r="J127" s="93" t="n"/>
+      <c r="K127" s="61" t="n"/>
+      <c r="L127" s="62" t="n"/>
+      <c r="M127" s="59">
         <f>IF(I127="","",ROUND(I127-E127,2))</f>
         <v/>
       </c>
-      <c r="L127" s="60">
+      <c r="N127" s="60">
         <f>IF(J127="","",J127-F127)</f>
         <v/>
       </c>
-      <c r="M127" s="56" t="n"/>
-      <c r="N127" s="56" t="n"/>
+      <c r="O127" s="56" t="n"/>
+      <c r="P127" s="56" t="n"/>
     </row>
     <row r="128" ht="15" customHeight="1" s="47">
       <c r="A128" s="54" t="n"/>
@@ -3992,18 +4285,20 @@
       <c r="E128" s="59" t="n"/>
       <c r="F128" s="60" t="n"/>
       <c r="G128" s="54" t="n"/>
-      <c r="I128" s="61" t="n"/>
-      <c r="J128" s="62" t="n"/>
-      <c r="K128" s="59">
+      <c r="I128" s="92" t="n"/>
+      <c r="J128" s="93" t="n"/>
+      <c r="K128" s="61" t="n"/>
+      <c r="L128" s="62" t="n"/>
+      <c r="M128" s="59">
         <f>IF(I128="","",ROUND(I128-E128,2))</f>
         <v/>
       </c>
-      <c r="L128" s="60">
+      <c r="N128" s="60">
         <f>IF(J128="","",J128-F128)</f>
         <v/>
       </c>
-      <c r="M128" s="56" t="n"/>
-      <c r="N128" s="56" t="n"/>
+      <c r="O128" s="56" t="n"/>
+      <c r="P128" s="56" t="n"/>
     </row>
     <row r="129" ht="15" customHeight="1" s="47">
       <c r="A129" s="54" t="n"/>
@@ -4013,18 +4308,20 @@
       <c r="E129" s="59" t="n"/>
       <c r="F129" s="60" t="n"/>
       <c r="G129" s="54" t="n"/>
-      <c r="I129" s="61" t="n"/>
-      <c r="J129" s="62" t="n"/>
-      <c r="K129" s="59">
+      <c r="I129" s="92" t="n"/>
+      <c r="J129" s="93" t="n"/>
+      <c r="K129" s="61" t="n"/>
+      <c r="L129" s="62" t="n"/>
+      <c r="M129" s="59">
         <f>IF(I129="","",ROUND(I129-E129,2))</f>
         <v/>
       </c>
-      <c r="L129" s="60">
+      <c r="N129" s="60">
         <f>IF(J129="","",J129-F129)</f>
         <v/>
       </c>
-      <c r="M129" s="56" t="n"/>
-      <c r="N129" s="56" t="n"/>
+      <c r="O129" s="56" t="n"/>
+      <c r="P129" s="56" t="n"/>
     </row>
     <row r="130" ht="15" customHeight="1" s="47">
       <c r="A130" s="54" t="n"/>
@@ -4034,18 +4331,20 @@
       <c r="E130" s="59" t="n"/>
       <c r="F130" s="60" t="n"/>
       <c r="G130" s="54" t="n"/>
-      <c r="I130" s="61" t="n"/>
-      <c r="J130" s="62" t="n"/>
-      <c r="K130" s="59">
+      <c r="I130" s="92" t="n"/>
+      <c r="J130" s="93" t="n"/>
+      <c r="K130" s="61" t="n"/>
+      <c r="L130" s="62" t="n"/>
+      <c r="M130" s="59">
         <f>IF(I130="","",ROUND(I130-E130,2))</f>
         <v/>
       </c>
-      <c r="L130" s="60">
+      <c r="N130" s="60">
         <f>IF(J130="","",J130-F130)</f>
         <v/>
       </c>
-      <c r="M130" s="56" t="n"/>
-      <c r="N130" s="56" t="n"/>
+      <c r="O130" s="56" t="n"/>
+      <c r="P130" s="56" t="n"/>
     </row>
     <row r="131" ht="15" customHeight="1" s="47">
       <c r="A131" s="54" t="n"/>
@@ -4055,18 +4354,20 @@
       <c r="E131" s="59" t="n"/>
       <c r="F131" s="60" t="n"/>
       <c r="G131" s="54" t="n"/>
-      <c r="I131" s="61" t="n"/>
-      <c r="J131" s="62" t="n"/>
-      <c r="K131" s="59">
+      <c r="I131" s="92" t="n"/>
+      <c r="J131" s="93" t="n"/>
+      <c r="K131" s="61" t="n"/>
+      <c r="L131" s="62" t="n"/>
+      <c r="M131" s="59">
         <f>IF(I131="","",ROUND(I131-E131,2))</f>
         <v/>
       </c>
-      <c r="L131" s="60">
+      <c r="N131" s="60">
         <f>IF(J131="","",J131-F131)</f>
         <v/>
       </c>
-      <c r="M131" s="56" t="n"/>
-      <c r="N131" s="56" t="n"/>
+      <c r="O131" s="56" t="n"/>
+      <c r="P131" s="56" t="n"/>
     </row>
     <row r="132" ht="15" customHeight="1" s="47">
       <c r="A132" s="54" t="n"/>
@@ -4076,18 +4377,20 @@
       <c r="E132" s="59" t="n"/>
       <c r="F132" s="60" t="n"/>
       <c r="G132" s="54" t="n"/>
-      <c r="I132" s="61" t="n"/>
-      <c r="J132" s="62" t="n"/>
-      <c r="K132" s="59">
+      <c r="I132" s="92" t="n"/>
+      <c r="J132" s="93" t="n"/>
+      <c r="K132" s="61" t="n"/>
+      <c r="L132" s="62" t="n"/>
+      <c r="M132" s="59">
         <f>IF(I132="","",ROUND(I132-E132,2))</f>
         <v/>
       </c>
-      <c r="L132" s="60">
+      <c r="N132" s="60">
         <f>IF(J132="","",J132-F132)</f>
         <v/>
       </c>
-      <c r="M132" s="56" t="n"/>
-      <c r="N132" s="56" t="n"/>
+      <c r="O132" s="56" t="n"/>
+      <c r="P132" s="56" t="n"/>
     </row>
     <row r="133" ht="15" customHeight="1" s="47">
       <c r="A133" s="54" t="n"/>
@@ -4097,18 +4400,20 @@
       <c r="E133" s="59" t="n"/>
       <c r="F133" s="60" t="n"/>
       <c r="G133" s="54" t="n"/>
-      <c r="I133" s="61" t="n"/>
-      <c r="J133" s="62" t="n"/>
-      <c r="K133" s="59">
+      <c r="I133" s="92" t="n"/>
+      <c r="J133" s="93" t="n"/>
+      <c r="K133" s="61" t="n"/>
+      <c r="L133" s="62" t="n"/>
+      <c r="M133" s="59">
         <f>IF(I133="","",ROUND(I133-E133,2))</f>
         <v/>
       </c>
-      <c r="L133" s="60">
+      <c r="N133" s="60">
         <f>IF(J133="","",J133-F133)</f>
         <v/>
       </c>
-      <c r="M133" s="56" t="n"/>
-      <c r="N133" s="56" t="n"/>
+      <c r="O133" s="56" t="n"/>
+      <c r="P133" s="56" t="n"/>
     </row>
     <row r="134" ht="15" customHeight="1" s="47">
       <c r="A134" s="54" t="n"/>
@@ -4118,18 +4423,20 @@
       <c r="E134" s="59" t="n"/>
       <c r="F134" s="60" t="n"/>
       <c r="G134" s="54" t="n"/>
-      <c r="I134" s="61" t="n"/>
-      <c r="J134" s="62" t="n"/>
-      <c r="K134" s="59">
+      <c r="I134" s="92" t="n"/>
+      <c r="J134" s="93" t="n"/>
+      <c r="K134" s="61" t="n"/>
+      <c r="L134" s="62" t="n"/>
+      <c r="M134" s="59">
         <f>IF(I134="","",ROUND(I134-E134,2))</f>
         <v/>
       </c>
-      <c r="L134" s="60">
+      <c r="N134" s="60">
         <f>IF(J134="","",J134-F134)</f>
         <v/>
       </c>
-      <c r="M134" s="56" t="n"/>
-      <c r="N134" s="56" t="n"/>
+      <c r="O134" s="56" t="n"/>
+      <c r="P134" s="56" t="n"/>
     </row>
     <row r="135" ht="15" customHeight="1" s="47">
       <c r="A135" s="54" t="n"/>
@@ -4139,18 +4446,20 @@
       <c r="E135" s="59" t="n"/>
       <c r="F135" s="60" t="n"/>
       <c r="G135" s="54" t="n"/>
-      <c r="I135" s="61" t="n"/>
-      <c r="J135" s="62" t="n"/>
-      <c r="K135" s="59">
+      <c r="I135" s="92" t="n"/>
+      <c r="J135" s="93" t="n"/>
+      <c r="K135" s="61" t="n"/>
+      <c r="L135" s="62" t="n"/>
+      <c r="M135" s="59">
         <f>IF(I135="","",ROUND(I135-E135,2))</f>
         <v/>
       </c>
-      <c r="L135" s="60">
+      <c r="N135" s="60">
         <f>IF(J135="","",J135-F135)</f>
         <v/>
       </c>
-      <c r="M135" s="56" t="n"/>
-      <c r="N135" s="56" t="n"/>
+      <c r="O135" s="56" t="n"/>
+      <c r="P135" s="56" t="n"/>
     </row>
     <row r="136" ht="15" customHeight="1" s="47">
       <c r="A136" s="54" t="n"/>
@@ -4160,18 +4469,20 @@
       <c r="E136" s="59" t="n"/>
       <c r="F136" s="60" t="n"/>
       <c r="G136" s="54" t="n"/>
-      <c r="I136" s="61" t="n"/>
-      <c r="J136" s="62" t="n"/>
-      <c r="K136" s="59">
+      <c r="I136" s="92" t="n"/>
+      <c r="J136" s="93" t="n"/>
+      <c r="K136" s="61" t="n"/>
+      <c r="L136" s="62" t="n"/>
+      <c r="M136" s="59">
         <f>IF(I136="","",ROUND(I136-E136,2))</f>
         <v/>
       </c>
-      <c r="L136" s="60">
+      <c r="N136" s="60">
         <f>IF(J136="","",J136-F136)</f>
         <v/>
       </c>
-      <c r="M136" s="56" t="n"/>
-      <c r="N136" s="56" t="n"/>
+      <c r="O136" s="56" t="n"/>
+      <c r="P136" s="56" t="n"/>
     </row>
     <row r="137" ht="15" customHeight="1" s="47">
       <c r="A137" s="54" t="n"/>
@@ -4181,18 +4492,20 @@
       <c r="E137" s="59" t="n"/>
       <c r="F137" s="60" t="n"/>
       <c r="G137" s="54" t="n"/>
-      <c r="I137" s="61" t="n"/>
-      <c r="J137" s="62" t="n"/>
-      <c r="K137" s="59">
+      <c r="I137" s="92" t="n"/>
+      <c r="J137" s="93" t="n"/>
+      <c r="K137" s="61" t="n"/>
+      <c r="L137" s="62" t="n"/>
+      <c r="M137" s="59">
         <f>IF(I137="","",ROUND(I137-E137,2))</f>
         <v/>
       </c>
-      <c r="L137" s="60">
+      <c r="N137" s="60">
         <f>IF(J137="","",J137-F137)</f>
         <v/>
       </c>
-      <c r="M137" s="56" t="n"/>
-      <c r="N137" s="56" t="n"/>
+      <c r="O137" s="56" t="n"/>
+      <c r="P137" s="56" t="n"/>
     </row>
     <row r="138" ht="15" customHeight="1" s="47">
       <c r="A138" s="54" t="n"/>
@@ -4202,18 +4515,20 @@
       <c r="E138" s="59" t="n"/>
       <c r="F138" s="60" t="n"/>
       <c r="G138" s="54" t="n"/>
-      <c r="I138" s="61" t="n"/>
-      <c r="J138" s="62" t="n"/>
-      <c r="K138" s="59">
+      <c r="I138" s="92" t="n"/>
+      <c r="J138" s="93" t="n"/>
+      <c r="K138" s="61" t="n"/>
+      <c r="L138" s="62" t="n"/>
+      <c r="M138" s="59">
         <f>IF(I138="","",ROUND(I138-E138,2))</f>
         <v/>
       </c>
-      <c r="L138" s="60">
+      <c r="N138" s="60">
         <f>IF(J138="","",J138-F138)</f>
         <v/>
       </c>
-      <c r="M138" s="56" t="n"/>
-      <c r="N138" s="56" t="n"/>
+      <c r="O138" s="56" t="n"/>
+      <c r="P138" s="56" t="n"/>
     </row>
     <row r="139" ht="15" customHeight="1" s="47">
       <c r="A139" s="54" t="n"/>
@@ -4223,18 +4538,20 @@
       <c r="E139" s="59" t="n"/>
       <c r="F139" s="60" t="n"/>
       <c r="G139" s="54" t="n"/>
-      <c r="I139" s="61" t="n"/>
-      <c r="J139" s="62" t="n"/>
-      <c r="K139" s="59">
+      <c r="I139" s="92" t="n"/>
+      <c r="J139" s="93" t="n"/>
+      <c r="K139" s="61" t="n"/>
+      <c r="L139" s="62" t="n"/>
+      <c r="M139" s="59">
         <f>IF(I139="","",ROUND(I139-E139,2))</f>
         <v/>
       </c>
-      <c r="L139" s="60">
+      <c r="N139" s="60">
         <f>IF(J139="","",J139-F139)</f>
         <v/>
       </c>
-      <c r="M139" s="56" t="n"/>
-      <c r="N139" s="56" t="n"/>
+      <c r="O139" s="56" t="n"/>
+      <c r="P139" s="56" t="n"/>
     </row>
     <row r="140" ht="15" customHeight="1" s="47">
       <c r="A140" s="54" t="n"/>
@@ -4244,18 +4561,20 @@
       <c r="E140" s="59" t="n"/>
       <c r="F140" s="60" t="n"/>
       <c r="G140" s="54" t="n"/>
-      <c r="I140" s="61" t="n"/>
-      <c r="J140" s="62" t="n"/>
-      <c r="K140" s="59">
+      <c r="I140" s="92" t="n"/>
+      <c r="J140" s="93" t="n"/>
+      <c r="K140" s="61" t="n"/>
+      <c r="L140" s="62" t="n"/>
+      <c r="M140" s="59">
         <f>IF(I140="","",ROUND(I140-E140,2))</f>
         <v/>
       </c>
-      <c r="L140" s="60">
+      <c r="N140" s="60">
         <f>IF(J140="","",J140-F140)</f>
         <v/>
       </c>
-      <c r="M140" s="56" t="n"/>
-      <c r="N140" s="56" t="n"/>
+      <c r="O140" s="56" t="n"/>
+      <c r="P140" s="56" t="n"/>
     </row>
     <row r="141" ht="15" customHeight="1" s="47">
       <c r="A141" s="54" t="n"/>
@@ -4265,18 +4584,20 @@
       <c r="E141" s="59" t="n"/>
       <c r="F141" s="60" t="n"/>
       <c r="G141" s="54" t="n"/>
-      <c r="I141" s="61" t="n"/>
-      <c r="J141" s="62" t="n"/>
-      <c r="K141" s="59">
+      <c r="I141" s="92" t="n"/>
+      <c r="J141" s="93" t="n"/>
+      <c r="K141" s="61" t="n"/>
+      <c r="L141" s="62" t="n"/>
+      <c r="M141" s="59">
         <f>IF(I141="","",ROUND(I141-E141,2))</f>
         <v/>
       </c>
-      <c r="L141" s="60">
+      <c r="N141" s="60">
         <f>IF(J141="","",J141-F141)</f>
         <v/>
       </c>
-      <c r="M141" s="56" t="n"/>
-      <c r="N141" s="56" t="n"/>
+      <c r="O141" s="56" t="n"/>
+      <c r="P141" s="56" t="n"/>
     </row>
     <row r="142" ht="15" customHeight="1" s="47">
       <c r="A142" s="54" t="n"/>
@@ -4286,18 +4607,20 @@
       <c r="E142" s="59" t="n"/>
       <c r="F142" s="60" t="n"/>
       <c r="G142" s="54" t="n"/>
-      <c r="I142" s="61" t="n"/>
-      <c r="J142" s="62" t="n"/>
-      <c r="K142" s="59">
+      <c r="I142" s="92" t="n"/>
+      <c r="J142" s="93" t="n"/>
+      <c r="K142" s="61" t="n"/>
+      <c r="L142" s="62" t="n"/>
+      <c r="M142" s="59">
         <f>IF(I142="","",ROUND(I142-E142,2))</f>
         <v/>
       </c>
-      <c r="L142" s="60">
+      <c r="N142" s="60">
         <f>IF(J142="","",J142-F142)</f>
         <v/>
       </c>
-      <c r="M142" s="56" t="n"/>
-      <c r="N142" s="56" t="n"/>
+      <c r="O142" s="56" t="n"/>
+      <c r="P142" s="56" t="n"/>
     </row>
     <row r="143" ht="15" customHeight="1" s="47">
       <c r="A143" s="54" t="n"/>
@@ -4307,18 +4630,20 @@
       <c r="E143" s="59" t="n"/>
       <c r="F143" s="60" t="n"/>
       <c r="G143" s="54" t="n"/>
-      <c r="I143" s="61" t="n"/>
-      <c r="J143" s="62" t="n"/>
-      <c r="K143" s="59">
+      <c r="I143" s="92" t="n"/>
+      <c r="J143" s="93" t="n"/>
+      <c r="K143" s="61" t="n"/>
+      <c r="L143" s="62" t="n"/>
+      <c r="M143" s="59">
         <f>IF(I143="","",ROUND(I143-E143,2))</f>
         <v/>
       </c>
-      <c r="L143" s="60">
+      <c r="N143" s="60">
         <f>IF(J143="","",J143-F143)</f>
         <v/>
       </c>
-      <c r="M143" s="56" t="n"/>
-      <c r="N143" s="56" t="n"/>
+      <c r="O143" s="56" t="n"/>
+      <c r="P143" s="56" t="n"/>
     </row>
     <row r="144" ht="15" customHeight="1" s="47">
       <c r="A144" s="54" t="n"/>
@@ -4328,18 +4653,20 @@
       <c r="E144" s="59" t="n"/>
       <c r="F144" s="60" t="n"/>
       <c r="G144" s="54" t="n"/>
-      <c r="I144" s="61" t="n"/>
-      <c r="J144" s="62" t="n"/>
-      <c r="K144" s="59">
+      <c r="I144" s="92" t="n"/>
+      <c r="J144" s="93" t="n"/>
+      <c r="K144" s="61" t="n"/>
+      <c r="L144" s="62" t="n"/>
+      <c r="M144" s="59">
         <f>IF(I144="","",ROUND(I144-E144,2))</f>
         <v/>
       </c>
-      <c r="L144" s="60">
+      <c r="N144" s="60">
         <f>IF(J144="","",J144-F144)</f>
         <v/>
       </c>
-      <c r="M144" s="56" t="n"/>
-      <c r="N144" s="56" t="n"/>
+      <c r="O144" s="56" t="n"/>
+      <c r="P144" s="56" t="n"/>
     </row>
     <row r="145" ht="15" customHeight="1" s="47">
       <c r="A145" s="54" t="n"/>
@@ -4349,18 +4676,20 @@
       <c r="E145" s="59" t="n"/>
       <c r="F145" s="60" t="n"/>
       <c r="G145" s="54" t="n"/>
-      <c r="I145" s="61" t="n"/>
-      <c r="J145" s="62" t="n"/>
-      <c r="K145" s="59">
+      <c r="I145" s="92" t="n"/>
+      <c r="J145" s="93" t="n"/>
+      <c r="K145" s="61" t="n"/>
+      <c r="L145" s="62" t="n"/>
+      <c r="M145" s="59">
         <f>IF(I145="","",ROUND(I145-E145,2))</f>
         <v/>
       </c>
-      <c r="L145" s="60">
+      <c r="N145" s="60">
         <f>IF(J145="","",J145-F145)</f>
         <v/>
       </c>
-      <c r="M145" s="56" t="n"/>
-      <c r="N145" s="56" t="n"/>
+      <c r="O145" s="56" t="n"/>
+      <c r="P145" s="56" t="n"/>
     </row>
     <row r="146" ht="15" customHeight="1" s="47">
       <c r="A146" s="54" t="n"/>
@@ -4370,18 +4699,20 @@
       <c r="E146" s="59" t="n"/>
       <c r="F146" s="60" t="n"/>
       <c r="G146" s="54" t="n"/>
-      <c r="I146" s="61" t="n"/>
-      <c r="J146" s="62" t="n"/>
-      <c r="K146" s="59">
+      <c r="I146" s="92" t="n"/>
+      <c r="J146" s="93" t="n"/>
+      <c r="K146" s="61" t="n"/>
+      <c r="L146" s="62" t="n"/>
+      <c r="M146" s="59">
         <f>IF(I146="","",ROUND(I146-E146,2))</f>
         <v/>
       </c>
-      <c r="L146" s="60">
+      <c r="N146" s="60">
         <f>IF(J146="","",J146-F146)</f>
         <v/>
       </c>
-      <c r="M146" s="56" t="n"/>
-      <c r="N146" s="56" t="n"/>
+      <c r="O146" s="56" t="n"/>
+      <c r="P146" s="56" t="n"/>
     </row>
     <row r="147" ht="15" customHeight="1" s="47">
       <c r="A147" s="54" t="n"/>
@@ -4391,18 +4722,20 @@
       <c r="E147" s="59" t="n"/>
       <c r="F147" s="60" t="n"/>
       <c r="G147" s="54" t="n"/>
-      <c r="I147" s="61" t="n"/>
-      <c r="J147" s="62" t="n"/>
-      <c r="K147" s="59">
+      <c r="I147" s="92" t="n"/>
+      <c r="J147" s="93" t="n"/>
+      <c r="K147" s="61" t="n"/>
+      <c r="L147" s="62" t="n"/>
+      <c r="M147" s="59">
         <f>IF(I147="","",ROUND(I147-E147,2))</f>
         <v/>
       </c>
-      <c r="L147" s="60">
+      <c r="N147" s="60">
         <f>IF(J147="","",J147-F147)</f>
         <v/>
       </c>
-      <c r="M147" s="56" t="n"/>
-      <c r="N147" s="56" t="n"/>
+      <c r="O147" s="56" t="n"/>
+      <c r="P147" s="56" t="n"/>
     </row>
     <row r="148" ht="15" customHeight="1" s="47">
       <c r="A148" s="54" t="n"/>
@@ -4412,18 +4745,20 @@
       <c r="E148" s="59" t="n"/>
       <c r="F148" s="60" t="n"/>
       <c r="G148" s="54" t="n"/>
-      <c r="I148" s="61" t="n"/>
-      <c r="J148" s="62" t="n"/>
-      <c r="K148" s="59">
+      <c r="I148" s="92" t="n"/>
+      <c r="J148" s="93" t="n"/>
+      <c r="K148" s="61" t="n"/>
+      <c r="L148" s="62" t="n"/>
+      <c r="M148" s="59">
         <f>IF(I148="","",ROUND(I148-E148,2))</f>
         <v/>
       </c>
-      <c r="L148" s="60">
+      <c r="N148" s="60">
         <f>IF(J148="","",J148-F148)</f>
         <v/>
       </c>
-      <c r="M148" s="56" t="n"/>
-      <c r="N148" s="56" t="n"/>
+      <c r="O148" s="56" t="n"/>
+      <c r="P148" s="56" t="n"/>
     </row>
     <row r="149" ht="15" customHeight="1" s="47">
       <c r="A149" s="54" t="n"/>
@@ -4433,18 +4768,20 @@
       <c r="E149" s="59" t="n"/>
       <c r="F149" s="60" t="n"/>
       <c r="G149" s="54" t="n"/>
-      <c r="I149" s="61" t="n"/>
-      <c r="J149" s="62" t="n"/>
-      <c r="K149" s="59">
+      <c r="I149" s="92" t="n"/>
+      <c r="J149" s="93" t="n"/>
+      <c r="K149" s="61" t="n"/>
+      <c r="L149" s="62" t="n"/>
+      <c r="M149" s="59">
         <f>IF(I149="","",ROUND(I149-E149,2))</f>
         <v/>
       </c>
-      <c r="L149" s="60">
+      <c r="N149" s="60">
         <f>IF(J149="","",J149-F149)</f>
         <v/>
       </c>
-      <c r="M149" s="56" t="n"/>
-      <c r="N149" s="56" t="n"/>
+      <c r="O149" s="56" t="n"/>
+      <c r="P149" s="56" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1" s="47">
       <c r="A150" s="54" t="n"/>
@@ -4454,18 +4791,20 @@
       <c r="E150" s="59" t="n"/>
       <c r="F150" s="60" t="n"/>
       <c r="G150" s="54" t="n"/>
-      <c r="I150" s="61" t="n"/>
-      <c r="J150" s="62" t="n"/>
-      <c r="K150" s="59">
+      <c r="I150" s="92" t="n"/>
+      <c r="J150" s="93" t="n"/>
+      <c r="K150" s="61" t="n"/>
+      <c r="L150" s="62" t="n"/>
+      <c r="M150" s="59">
         <f>IF(I150="","",ROUND(I150-E150,2))</f>
         <v/>
       </c>
-      <c r="L150" s="60">
+      <c r="N150" s="60">
         <f>IF(J150="","",J150-F150)</f>
         <v/>
       </c>
-      <c r="M150" s="56" t="n"/>
-      <c r="N150" s="56" t="n"/>
+      <c r="O150" s="56" t="n"/>
+      <c r="P150" s="56" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1" s="47">
       <c r="A151" s="54" t="n"/>
@@ -4475,18 +4814,20 @@
       <c r="E151" s="59" t="n"/>
       <c r="F151" s="60" t="n"/>
       <c r="G151" s="54" t="n"/>
-      <c r="I151" s="61" t="n"/>
-      <c r="J151" s="62" t="n"/>
-      <c r="K151" s="59">
+      <c r="I151" s="92" t="n"/>
+      <c r="J151" s="93" t="n"/>
+      <c r="K151" s="61" t="n"/>
+      <c r="L151" s="62" t="n"/>
+      <c r="M151" s="59">
         <f>IF(I151="","",ROUND(I151-E151,2))</f>
         <v/>
       </c>
-      <c r="L151" s="60">
+      <c r="N151" s="60">
         <f>IF(J151="","",J151-F151)</f>
         <v/>
       </c>
-      <c r="M151" s="56" t="n"/>
-      <c r="N151" s="56" t="n"/>
+      <c r="O151" s="56" t="n"/>
+      <c r="P151" s="56" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1" s="47">
       <c r="A152" s="54" t="n"/>
@@ -4496,18 +4837,20 @@
       <c r="E152" s="59" t="n"/>
       <c r="F152" s="60" t="n"/>
       <c r="G152" s="54" t="n"/>
-      <c r="I152" s="61" t="n"/>
-      <c r="J152" s="62" t="n"/>
-      <c r="K152" s="59">
+      <c r="I152" s="92" t="n"/>
+      <c r="J152" s="93" t="n"/>
+      <c r="K152" s="61" t="n"/>
+      <c r="L152" s="62" t="n"/>
+      <c r="M152" s="59">
         <f>IF(I152="","",ROUND(I152-E152,2))</f>
         <v/>
       </c>
-      <c r="L152" s="60">
+      <c r="N152" s="60">
         <f>IF(J152="","",J152-F152)</f>
         <v/>
       </c>
-      <c r="M152" s="56" t="n"/>
-      <c r="N152" s="56" t="n"/>
+      <c r="O152" s="56" t="n"/>
+      <c r="P152" s="56" t="n"/>
     </row>
     <row r="153" ht="15" customHeight="1" s="47">
       <c r="A153" s="54" t="n"/>
@@ -4517,18 +4860,20 @@
       <c r="E153" s="59" t="n"/>
       <c r="F153" s="60" t="n"/>
       <c r="G153" s="54" t="n"/>
-      <c r="I153" s="61" t="n"/>
-      <c r="J153" s="62" t="n"/>
-      <c r="K153" s="59">
+      <c r="I153" s="92" t="n"/>
+      <c r="J153" s="93" t="n"/>
+      <c r="K153" s="61" t="n"/>
+      <c r="L153" s="62" t="n"/>
+      <c r="M153" s="59">
         <f>IF(I153="","",ROUND(I153-E153,2))</f>
         <v/>
       </c>
-      <c r="L153" s="60">
+      <c r="N153" s="60">
         <f>IF(J153="","",J153-F153)</f>
         <v/>
       </c>
-      <c r="M153" s="56" t="n"/>
-      <c r="N153" s="56" t="n"/>
+      <c r="O153" s="56" t="n"/>
+      <c r="P153" s="56" t="n"/>
     </row>
     <row r="154" ht="15" customHeight="1" s="47">
       <c r="A154" s="54" t="n"/>
@@ -4538,18 +4883,20 @@
       <c r="E154" s="59" t="n"/>
       <c r="F154" s="60" t="n"/>
       <c r="G154" s="54" t="n"/>
-      <c r="I154" s="61" t="n"/>
-      <c r="J154" s="62" t="n"/>
-      <c r="K154" s="59">
+      <c r="I154" s="92" t="n"/>
+      <c r="J154" s="93" t="n"/>
+      <c r="K154" s="61" t="n"/>
+      <c r="L154" s="62" t="n"/>
+      <c r="M154" s="59">
         <f>IF(I154="","",ROUND(I154-E154,2))</f>
         <v/>
       </c>
-      <c r="L154" s="60">
+      <c r="N154" s="60">
         <f>IF(J154="","",J154-F154)</f>
         <v/>
       </c>
-      <c r="M154" s="56" t="n"/>
-      <c r="N154" s="56" t="n"/>
+      <c r="O154" s="56" t="n"/>
+      <c r="P154" s="56" t="n"/>
     </row>
     <row r="155" ht="15" customHeight="1" s="47">
       <c r="A155" s="54" t="n"/>
@@ -4559,18 +4906,20 @@
       <c r="E155" s="59" t="n"/>
       <c r="F155" s="60" t="n"/>
       <c r="G155" s="54" t="n"/>
-      <c r="I155" s="61" t="n"/>
-      <c r="J155" s="62" t="n"/>
-      <c r="K155" s="59">
+      <c r="I155" s="92" t="n"/>
+      <c r="J155" s="93" t="n"/>
+      <c r="K155" s="61" t="n"/>
+      <c r="L155" s="62" t="n"/>
+      <c r="M155" s="59">
         <f>IF(I155="","",ROUND(I155-E155,2))</f>
         <v/>
       </c>
-      <c r="L155" s="60">
+      <c r="N155" s="60">
         <f>IF(J155="","",J155-F155)</f>
         <v/>
       </c>
-      <c r="M155" s="56" t="n"/>
-      <c r="N155" s="56" t="n"/>
+      <c r="O155" s="56" t="n"/>
+      <c r="P155" s="56" t="n"/>
     </row>
     <row r="156" ht="15" customHeight="1" s="47">
       <c r="A156" s="54" t="n"/>
@@ -4580,18 +4929,20 @@
       <c r="E156" s="59" t="n"/>
       <c r="F156" s="60" t="n"/>
       <c r="G156" s="54" t="n"/>
-      <c r="I156" s="61" t="n"/>
-      <c r="J156" s="62" t="n"/>
-      <c r="K156" s="59">
+      <c r="I156" s="92" t="n"/>
+      <c r="J156" s="93" t="n"/>
+      <c r="K156" s="61" t="n"/>
+      <c r="L156" s="62" t="n"/>
+      <c r="M156" s="59">
         <f>IF(I156="","",ROUND(I156-E156,2))</f>
         <v/>
       </c>
-      <c r="L156" s="60">
+      <c r="N156" s="60">
         <f>IF(J156="","",J156-F156)</f>
         <v/>
       </c>
-      <c r="M156" s="56" t="n"/>
-      <c r="N156" s="56" t="n"/>
+      <c r="O156" s="56" t="n"/>
+      <c r="P156" s="56" t="n"/>
     </row>
     <row r="157" ht="15" customHeight="1" s="47">
       <c r="A157" s="54" t="n"/>
@@ -4601,18 +4952,20 @@
       <c r="E157" s="59" t="n"/>
       <c r="F157" s="60" t="n"/>
       <c r="G157" s="54" t="n"/>
-      <c r="I157" s="61" t="n"/>
-      <c r="J157" s="62" t="n"/>
-      <c r="K157" s="59">
+      <c r="I157" s="92" t="n"/>
+      <c r="J157" s="93" t="n"/>
+      <c r="K157" s="61" t="n"/>
+      <c r="L157" s="62" t="n"/>
+      <c r="M157" s="59">
         <f>IF(I157="","",ROUND(I157-E157,2))</f>
         <v/>
       </c>
-      <c r="L157" s="60">
+      <c r="N157" s="60">
         <f>IF(J157="","",J157-F157)</f>
         <v/>
       </c>
-      <c r="M157" s="56" t="n"/>
-      <c r="N157" s="56" t="n"/>
+      <c r="O157" s="56" t="n"/>
+      <c r="P157" s="56" t="n"/>
     </row>
     <row r="158" ht="15" customHeight="1" s="47">
       <c r="A158" s="54" t="n"/>
@@ -4622,18 +4975,20 @@
       <c r="E158" s="59" t="n"/>
       <c r="F158" s="60" t="n"/>
       <c r="G158" s="54" t="n"/>
-      <c r="I158" s="61" t="n"/>
-      <c r="J158" s="62" t="n"/>
-      <c r="K158" s="59">
+      <c r="I158" s="92" t="n"/>
+      <c r="J158" s="93" t="n"/>
+      <c r="K158" s="61" t="n"/>
+      <c r="L158" s="62" t="n"/>
+      <c r="M158" s="59">
         <f>IF(I158="","",ROUND(I158-E158,2))</f>
         <v/>
       </c>
-      <c r="L158" s="60">
+      <c r="N158" s="60">
         <f>IF(J158="","",J158-F158)</f>
         <v/>
       </c>
-      <c r="M158" s="56" t="n"/>
-      <c r="N158" s="56" t="n"/>
+      <c r="O158" s="56" t="n"/>
+      <c r="P158" s="56" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1" s="47">
       <c r="A159" s="54" t="n"/>
@@ -4643,18 +4998,20 @@
       <c r="E159" s="59" t="n"/>
       <c r="F159" s="60" t="n"/>
       <c r="G159" s="54" t="n"/>
-      <c r="I159" s="61" t="n"/>
-      <c r="J159" s="62" t="n"/>
-      <c r="K159" s="59">
+      <c r="I159" s="92" t="n"/>
+      <c r="J159" s="93" t="n"/>
+      <c r="K159" s="61" t="n"/>
+      <c r="L159" s="62" t="n"/>
+      <c r="M159" s="59">
         <f>IF(I159="","",ROUND(I159-E159,2))</f>
         <v/>
       </c>
-      <c r="L159" s="60">
+      <c r="N159" s="60">
         <f>IF(J159="","",J159-F159)</f>
         <v/>
       </c>
-      <c r="M159" s="56" t="n"/>
-      <c r="N159" s="56" t="n"/>
+      <c r="O159" s="56" t="n"/>
+      <c r="P159" s="56" t="n"/>
     </row>
     <row r="160" ht="15" customHeight="1" s="47">
       <c r="A160" s="54" t="n"/>
@@ -4664,18 +5021,20 @@
       <c r="E160" s="59" t="n"/>
       <c r="F160" s="60" t="n"/>
       <c r="G160" s="54" t="n"/>
-      <c r="I160" s="61" t="n"/>
-      <c r="J160" s="62" t="n"/>
-      <c r="K160" s="59">
+      <c r="I160" s="92" t="n"/>
+      <c r="J160" s="93" t="n"/>
+      <c r="K160" s="61" t="n"/>
+      <c r="L160" s="62" t="n"/>
+      <c r="M160" s="59">
         <f>IF(I160="","",ROUND(I160-E160,2))</f>
         <v/>
       </c>
-      <c r="L160" s="60">
+      <c r="N160" s="60">
         <f>IF(J160="","",J160-F160)</f>
         <v/>
       </c>
-      <c r="M160" s="56" t="n"/>
-      <c r="N160" s="56" t="n"/>
+      <c r="O160" s="56" t="n"/>
+      <c r="P160" s="56" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1" s="47">
       <c r="A161" s="63" t="n"/>
@@ -4695,24 +5054,26 @@
         <v/>
       </c>
       <c r="G161" s="63" t="n"/>
-      <c r="I161" s="65">
+      <c r="I161" s="92" t="n"/>
+      <c r="J161" s="93" t="n"/>
+      <c r="K161" s="65">
         <f>SUM(I5:I160)</f>
         <v/>
       </c>
-      <c r="J161" s="66">
+      <c r="L161" s="66">
         <f>SUM(J5:J160)</f>
         <v/>
       </c>
-      <c r="K161" s="65">
+      <c r="M161" s="65">
         <f>SUM(K5:K160)</f>
         <v/>
       </c>
-      <c r="L161" s="66">
+      <c r="N161" s="66">
         <f>SUM(L5:L160)</f>
         <v/>
       </c>
-      <c r="M161" s="63" t="n"/>
-      <c r="N161" s="63" t="n"/>
+      <c r="O161" s="63" t="n"/>
+      <c r="P161" s="63" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:M160"/>
@@ -20276,11 +20637,11 @@
         <v/>
       </c>
       <c r="F5" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A5,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A5,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G5" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A5,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A5,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H5" s="59">
@@ -20324,11 +20685,11 @@
         <v/>
       </c>
       <c r="F6" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A6,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A6,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G6" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A6,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A6,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H6" s="59">
@@ -20372,11 +20733,11 @@
         <v/>
       </c>
       <c r="F7" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A7,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A7,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G7" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A7,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A7,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H7" s="59">
@@ -20420,11 +20781,11 @@
         <v/>
       </c>
       <c r="F8" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A8,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A8,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G8" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A8,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A8,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H8" s="59">
@@ -20468,11 +20829,11 @@
         <v/>
       </c>
       <c r="F9" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A9,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A9,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G9" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A9,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A9,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H9" s="59">
@@ -20516,11 +20877,11 @@
         <v/>
       </c>
       <c r="F10" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A10,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A10,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G10" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A10,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A10,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H10" s="59">
@@ -20564,11 +20925,11 @@
         <v/>
       </c>
       <c r="F11" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A11,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A11,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G11" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A11,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A11,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H11" s="59">
@@ -20612,11 +20973,11 @@
         <v/>
       </c>
       <c r="F12" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A12,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A12,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G12" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A12,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A12,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H12" s="59">
@@ -20660,11 +21021,11 @@
         <v/>
       </c>
       <c r="F13" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A13,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A13,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G13" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A13,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A13,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H13" s="59">
@@ -20708,11 +21069,11 @@
         <v/>
       </c>
       <c r="F14" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A14,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A14,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G14" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A14,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A14,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H14" s="59">
@@ -20756,11 +21117,11 @@
         <v/>
       </c>
       <c r="F15" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A15,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A15,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G15" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A15,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A15,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H15" s="59">
@@ -20804,11 +21165,11 @@
         <v/>
       </c>
       <c r="F16" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A16,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A16,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G16" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A16,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A16,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H16" s="59">
@@ -20852,11 +21213,11 @@
         <v/>
       </c>
       <c r="F17" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A17,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A17,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G17" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A17,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A17,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H17" s="59">
@@ -20900,11 +21261,11 @@
         <v/>
       </c>
       <c r="F18" s="59">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A18,'Count Sheet'!$I$5:$I$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A18,'Count Sheet'!$K$5:$K$160)</f>
         <v/>
       </c>
       <c r="G18" s="60">
-        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A18,'Count Sheet'!$J$5:$J$160)</f>
+        <f>SUMIF('Count Sheet'!$A$5:$A$160,$A18,'Count Sheet'!$L$5:$L$160)</f>
         <v/>
       </c>
       <c r="H18" s="59">

</xml_diff>